<commit_message>
Add Kia Picanto TO kit (TO-13) with user's supplier prices
- kits.json: TO-13 Kia Picanto 1.0/1.2 with Hyundai/Kia 5W-30 4 L oil,
  oil/air/cabin filters, drain washer and repair card
- listing photos and repair card generated for the kit
- workbook regenerated with TO-13 rows; brands pre-filled and the
  quoted purchase prices noted per line for the user to enter under
  the right supplier; oil spec check note (SM/GF-4+ recommended)
- listings.md: ready-to-paste Picanto listing (price 4 190 ₽ from
  3 225,70 ₽ purchase incl. washer estimate and packaging)
- docs: kit counts updated to 24 (13 TO + 11 GRM)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="254">
   <si>
     <t xml:space="preserve">ZAPKIT — таблица закупки и цен</t>
   </si>
@@ -334,6 +334,21 @@
     <t xml:space="preserve">to-12-coolray-1-main.png</t>
   </si>
   <si>
+    <t xml:space="preserve">TO-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kia Picanto 1.0 / 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G3LA 1.0 / G4LA 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТО-кит Kia Picanto 1.0/1.2: масло и фильтры</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to-13-picanto-1-main.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">GRM-01</t>
   </si>
   <si>
@@ -578,6 +593,30 @@
   </si>
   <si>
     <t xml:space="preserve">Поставьте 1, если объём заливки с фильтром больше 4 л (проверьте по VIN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyundai/Kia Super Extra Gasoline 5W-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 2 051,00 ₽ — впишите в колонку поставщика, у которого брали. Проверьте допуск: для Picanto рекомендуют API SM / ILSAC GF-4 и выше.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 154,70 ₽ — впишите в колонку поставщика, у которого брали.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 533,00 ₽ — впишите в колонку поставщика, у которого брали.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIG FILTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 387,00 ₽ — впишите в колонку поставщика, у которого брали.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Добавлена по стандартному составу ТО-кита; подберите по VIN (обычно 30–60 ₽).</t>
   </si>
   <si>
     <t xml:space="preserve">Комплект цепи ГРМ (цепь, натяжитель, успокоители)</t>
@@ -1394,7 +1433,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -2118,13 +2157,13 @@
         <v>91</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>30</v>
-      </c>
       <c r="D14" s="7" t="s">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>32</v>
@@ -2133,10 +2172,10 @@
         <v>33</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A14)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A14)+Параметры!$B$3)</f>
@@ -2144,7 +2183,7 @@
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A14,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K14" s="11" t="str">
         <f aca="false">IF(I14="","",CEILING(I14*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2169,16 +2208,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>32</v>
@@ -2187,10 +2226,10 @@
         <v>33</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I15" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A15)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A15)+Параметры!$B$3)</f>
@@ -2223,16 +2262,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>32</v>
@@ -2241,10 +2280,10 @@
         <v>33</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I16" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A16)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A16)+Параметры!$B$3)</f>
@@ -2277,16 +2316,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>32</v>
@@ -2295,10 +2334,10 @@
         <v>33</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I17" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A17)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A17)+Параметры!$B$3)</f>
@@ -2331,28 +2370,28 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I18" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A18)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A18)+Параметры!$B$3)</f>
@@ -2385,28 +2424,28 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I19" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A19)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A19)+Параметры!$B$3)</f>
@@ -2414,7 +2453,7 @@
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A19,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K19" s="11" t="str">
         <f aca="false">IF(I19="","",CEILING(I19*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2439,28 +2478,28 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I20" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A20)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A20)+Параметры!$B$3)</f>
@@ -2468,7 +2507,7 @@
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A20,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K20" s="11" t="str">
         <f aca="false">IF(I20="","",CEILING(I20*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2493,28 +2532,28 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I21" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A21)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A21)+Параметры!$B$3)</f>
@@ -2547,28 +2586,28 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I22" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A22)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A22)+Параметры!$B$3)</f>
@@ -2601,22 +2640,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>121</v>
+        <v>72</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>123</v>
@@ -2658,25 +2697,25 @@
         <v>125</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>86</v>
+        <v>126</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>33</v>
+        <v>127</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I24" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A24)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A24)+Параметры!$B$3)</f>
@@ -2684,7 +2723,7 @@
       </c>
       <c r="J24" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A24,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K24" s="11" t="str">
         <f aca="false">IF(I24="","",CEILING(I24*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2707,19 +2746,73 @@
         <v>36</v>
       </c>
     </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="I25" s="9" t="str">
+        <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A25)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A25)+Параметры!$B$3)</f>
+        <v/>
+      </c>
+      <c r="J25" s="10" t="n">
+        <f aca="false">COUNTIFS(Состав!$A:$A,A25,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
+        <v>2</v>
+      </c>
+      <c r="K25" s="11" t="str">
+        <f aca="false">IF(I25="","",CEILING(I25*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
+        <v/>
+      </c>
+      <c r="L25" s="12"/>
+      <c r="M25" s="7" t="str">
+        <f aca="false">IF(OR(K25="",L25=""),"",IF(K25&lt;=L25,"не дороже рынка","дороже рынка"))</f>
+        <v/>
+      </c>
+      <c r="N25" s="9" t="str">
+        <f aca="false">IF(K25="","",K25-I25-K25*Параметры!$B$6-Параметры!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O25" s="13" t="str">
+        <f aca="false">IF(N25="","",N25/K25)</f>
+        <v/>
+      </c>
+      <c r="P25" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J2:J24">
+  <conditionalFormatting sqref="J2:J25">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M24">
+  <conditionalFormatting sqref="M2:M25">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"дороже рынка"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P24" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P25" type="list">
       <formula1>"не выложен,выложен,есть продажи,снят"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2750,79 +2843,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B2" s="15" t="n">
         <v>0.3</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>50</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>100</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>0.065</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>180</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2841,7 +2934,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S120"/>
+  <dimension ref="A1:S125"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -2865,75 +2958,75 @@
         <v>14</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D2" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="G2" s="19" t="n">
         <v>460</v>
@@ -2965,7 +3058,7 @@
         <v>430</v>
       </c>
       <c r="S2" s="21" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2977,7 +3070,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>1</v>
@@ -3006,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3018,7 +3111,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D4" s="14" t="n">
         <v>1</v>
@@ -3057,7 +3150,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>1</v>
@@ -3096,7 +3189,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>1</v>
@@ -3135,7 +3228,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>1</v>
@@ -3174,7 +3267,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D8" s="14" t="n">
         <v>1</v>
@@ -3203,7 +3296,7 @@
         <v>0</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3215,7 +3308,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>1</v>
@@ -3254,7 +3347,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>1</v>
@@ -3293,7 +3386,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>1</v>
@@ -3332,7 +3425,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>1</v>
@@ -3371,7 +3464,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>1</v>
@@ -3400,7 +3493,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3412,7 +3505,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D14" s="14" t="n">
         <v>1</v>
@@ -3451,7 +3544,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>1</v>
@@ -3490,7 +3583,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>1</v>
@@ -3529,7 +3622,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>1</v>
@@ -3568,7 +3661,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>1</v>
@@ -3597,7 +3690,7 @@
         <v>0</v>
       </c>
       <c r="S18" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3609,7 +3702,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>1</v>
@@ -3648,7 +3741,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D20" s="14" t="n">
         <v>1</v>
@@ -3687,7 +3780,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D21" s="14" t="n">
         <v>1</v>
@@ -3726,7 +3819,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D22" s="14" t="n">
         <v>1</v>
@@ -3765,7 +3858,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D23" s="14" t="n">
         <v>1</v>
@@ -3794,7 +3887,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,7 +3899,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D24" s="14" t="n">
         <v>1</v>
@@ -3845,7 +3938,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D25" s="14" t="n">
         <v>1</v>
@@ -3884,7 +3977,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D26" s="14" t="n">
         <v>1</v>
@@ -3923,7 +4016,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D27" s="14" t="n">
         <v>1</v>
@@ -3962,7 +4055,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D28" s="14" t="n">
         <v>1</v>
@@ -3991,7 +4084,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4003,7 +4096,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D29" s="14" t="n">
         <v>1</v>
@@ -4042,7 +4135,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D30" s="14" t="n">
         <v>1</v>
@@ -4081,7 +4174,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D31" s="14" t="n">
         <v>1</v>
@@ -4120,7 +4213,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D32" s="14" t="n">
         <v>1</v>
@@ -4159,7 +4252,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D33" s="14" t="n">
         <v>1</v>
@@ -4188,7 +4281,7 @@
         <v>0</v>
       </c>
       <c r="S33" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4200,7 +4293,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D34" s="14" t="n">
         <v>0</v>
@@ -4229,7 +4322,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4241,7 +4334,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D35" s="14" t="n">
         <v>1</v>
@@ -4280,7 +4373,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>1</v>
@@ -4319,7 +4412,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D37" s="14" t="n">
         <v>1</v>
@@ -4358,7 +4451,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D38" s="14" t="n">
         <v>1</v>
@@ -4397,7 +4490,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D39" s="14" t="n">
         <v>1</v>
@@ -4426,7 +4519,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4438,7 +4531,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>0</v>
@@ -4467,7 +4560,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4479,7 +4572,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D41" s="14" t="n">
         <v>1</v>
@@ -4518,7 +4611,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D42" s="14" t="n">
         <v>1</v>
@@ -4557,7 +4650,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D43" s="14" t="n">
         <v>1</v>
@@ -4596,7 +4689,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D44" s="14" t="n">
         <v>1</v>
@@ -4635,7 +4728,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D45" s="14" t="n">
         <v>1</v>
@@ -4664,7 +4757,7 @@
         <v>0</v>
       </c>
       <c r="S45" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4676,7 +4769,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D46" s="14" t="n">
         <v>0</v>
@@ -4705,7 +4798,7 @@
         <v>0</v>
       </c>
       <c r="S46" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4717,7 +4810,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D47" s="14" t="n">
         <v>1</v>
@@ -4756,7 +4849,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D48" s="14" t="n">
         <v>1</v>
@@ -4795,7 +4888,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D49" s="14" t="n">
         <v>1</v>
@@ -4834,7 +4927,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D50" s="14" t="n">
         <v>1</v>
@@ -4873,7 +4966,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D51" s="14" t="n">
         <v>1</v>
@@ -4902,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="S51" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4914,7 +5007,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D52" s="14" t="n">
         <v>0</v>
@@ -4943,7 +5036,7 @@
         <v>0</v>
       </c>
       <c r="S52" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4955,7 +5048,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D53" s="14" t="n">
         <v>1</v>
@@ -4994,7 +5087,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D54" s="14" t="n">
         <v>1</v>
@@ -5033,7 +5126,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D55" s="14" t="n">
         <v>1</v>
@@ -5072,7 +5165,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D56" s="14" t="n">
         <v>1</v>
@@ -5111,7 +5204,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D57" s="14" t="n">
         <v>1</v>
@@ -5140,7 +5233,7 @@
         <v>0</v>
       </c>
       <c r="S57" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5152,7 +5245,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D58" s="14" t="n">
         <v>0</v>
@@ -5181,7 +5274,7 @@
         <v>0</v>
       </c>
       <c r="S58" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5193,7 +5286,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D59" s="14" t="n">
         <v>1</v>
@@ -5232,7 +5325,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D60" s="14" t="n">
         <v>1</v>
@@ -5271,7 +5364,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D61" s="14" t="n">
         <v>1</v>
@@ -5310,7 +5403,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D62" s="14" t="n">
         <v>1</v>
@@ -5349,7 +5442,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D63" s="14" t="n">
         <v>1</v>
@@ -5378,7 +5471,7 @@
         <v>0</v>
       </c>
       <c r="S63" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5390,7 +5483,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D64" s="14" t="n">
         <v>0</v>
@@ -5419,7 +5512,7 @@
         <v>0</v>
       </c>
       <c r="S64" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5431,7 +5524,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D65" s="14" t="n">
         <v>1</v>
@@ -5470,7 +5563,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D66" s="14" t="n">
         <v>1</v>
@@ -5509,7 +5602,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D67" s="14" t="n">
         <v>1</v>
@@ -5548,7 +5641,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D68" s="14" t="n">
         <v>1</v>
@@ -5578,21 +5671,23 @@
       </c>
       <c r="S68" s="8"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
         <v>91</v>
       </c>
       <c r="B69" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A69,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D69" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E69" s="14"/>
+      <c r="E69" s="14" t="s">
+        <v>178</v>
+      </c>
       <c r="F69" s="14"/>
       <c r="G69" s="12"/>
       <c r="H69" s="12"/>
@@ -5616,7 +5711,7 @@
         <v>0</v>
       </c>
       <c r="S69" s="8" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5625,15 +5720,17 @@
       </c>
       <c r="B70" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A70,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="D70" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E70" s="14"/>
+      <c r="E70" s="14" t="s">
+        <v>180</v>
+      </c>
       <c r="F70" s="14"/>
       <c r="G70" s="12"/>
       <c r="H70" s="12"/>
@@ -5656,7 +5753,9 @@
         <f aca="false">IF(P70="",0,P70*D70)</f>
         <v>0</v>
       </c>
-      <c r="S70" s="8"/>
+      <c r="S70" s="8" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
@@ -5664,15 +5763,17 @@
       </c>
       <c r="B71" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A71,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D71" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E71" s="14"/>
+      <c r="E71" s="14" t="s">
+        <v>180</v>
+      </c>
       <c r="F71" s="14"/>
       <c r="G71" s="12"/>
       <c r="H71" s="12"/>
@@ -5695,7 +5796,9 @@
         <f aca="false">IF(P71="",0,P71*D71)</f>
         <v>0</v>
       </c>
-      <c r="S71" s="8"/>
+      <c r="S71" s="8" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
@@ -5703,15 +5806,17 @@
       </c>
       <c r="B72" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A72,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D72" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="14"/>
+        <v>1</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>183</v>
+      </c>
       <c r="F72" s="14"/>
       <c r="G72" s="12"/>
       <c r="H72" s="12"/>
@@ -5735,7 +5840,7 @@
         <v>0</v>
       </c>
       <c r="S72" s="8" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5744,13 +5849,13 @@
       </c>
       <c r="B73" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A73,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D73" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E73" s="14"/>
       <c r="F73" s="14"/>
@@ -5776,19 +5881,19 @@
         <v>0</v>
       </c>
       <c r="S73" s="8" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B74" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A74,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D74" s="14" t="n">
         <v>1</v>
@@ -5817,19 +5922,19 @@
         <v>0</v>
       </c>
       <c r="S74" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B75" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A75,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D75" s="14" t="n">
         <v>1</v>
@@ -5861,14 +5966,14 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B76" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A76,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D76" s="14" t="n">
         <v>1</v>
@@ -5900,14 +6005,14 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B77" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A77,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D77" s="14" t="n">
         <v>0</v>
@@ -5936,19 +6041,19 @@
         <v>0</v>
       </c>
       <c r="S77" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B78" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A78,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D78" s="14" t="n">
         <v>0</v>
@@ -5977,19 +6082,19 @@
         <v>0</v>
       </c>
       <c r="S78" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B79" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A79,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D79" s="14" t="n">
         <v>1</v>
@@ -6018,19 +6123,19 @@
         <v>0</v>
       </c>
       <c r="S79" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B80" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A80,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D80" s="14" t="n">
         <v>1</v>
@@ -6062,14 +6167,14 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B81" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A81,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D81" s="14" t="n">
         <v>1</v>
@@ -6101,14 +6206,14 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B82" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A82,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D82" s="14" t="n">
         <v>0</v>
@@ -6137,19 +6242,19 @@
         <v>0</v>
       </c>
       <c r="S82" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B83" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A83,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D83" s="14" t="n">
         <v>0</v>
@@ -6178,19 +6283,19 @@
         <v>0</v>
       </c>
       <c r="S83" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B84" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A84,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D84" s="14" t="n">
         <v>1</v>
@@ -6219,19 +6324,19 @@
         <v>0</v>
       </c>
       <c r="S84" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B85" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A85,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D85" s="14" t="n">
         <v>1</v>
@@ -6263,14 +6368,14 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B86" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A86,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D86" s="14" t="n">
         <v>1</v>
@@ -6302,14 +6407,14 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B87" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A87,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D87" s="14" t="n">
         <v>0</v>
@@ -6338,19 +6443,19 @@
         <v>0</v>
       </c>
       <c r="S87" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B88" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A88,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D88" s="14" t="n">
         <v>0</v>
@@ -6379,19 +6484,19 @@
         <v>0</v>
       </c>
       <c r="S88" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B89" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A89,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D89" s="14" t="n">
         <v>1</v>
@@ -6420,19 +6525,19 @@
         <v>0</v>
       </c>
       <c r="S89" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B90" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A90,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D90" s="14" t="n">
         <v>1</v>
@@ -6464,14 +6569,14 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B91" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A91,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D91" s="14" t="n">
         <v>1</v>
@@ -6503,14 +6608,14 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B92" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A92,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D92" s="14" t="n">
         <v>0</v>
@@ -6539,19 +6644,19 @@
         <v>0</v>
       </c>
       <c r="S92" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B93" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A93,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D93" s="14" t="n">
         <v>0</v>
@@ -6580,19 +6685,19 @@
         <v>0</v>
       </c>
       <c r="S93" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B94" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A94,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D94" s="14" t="n">
         <v>1</v>
@@ -6620,21 +6725,23 @@
         <f aca="false">IF(P94="",0,P94*D94)</f>
         <v>0</v>
       </c>
-      <c r="S94" s="8"/>
+      <c r="S94" s="8" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B95" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A95,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="D95" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E95" s="14"/>
       <c r="F95" s="14"/>
@@ -6659,23 +6766,21 @@
         <f aca="false">IF(P95="",0,P95*D95)</f>
         <v>0</v>
       </c>
-      <c r="S95" s="8" t="s">
-        <v>178</v>
-      </c>
+      <c r="S95" s="8"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B96" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A96,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="D96" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E96" s="14"/>
       <c r="F96" s="14"/>
@@ -6700,23 +6805,21 @@
         <f aca="false">IF(P96="",0,P96*D96)</f>
         <v>0</v>
       </c>
-      <c r="S96" s="8" t="s">
-        <v>180</v>
-      </c>
+      <c r="S96" s="8"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B97" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A97,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="D97" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" s="14"/>
       <c r="F97" s="14"/>
@@ -6742,22 +6845,22 @@
         <v>0</v>
       </c>
       <c r="S97" s="8" t="s">
-        <v>174</v>
+        <v>191</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B98" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A98,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="D98" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E98" s="14"/>
       <c r="F98" s="14"/>
@@ -6782,18 +6885,20 @@
         <f aca="false">IF(P98="",0,P98*D98)</f>
         <v>0</v>
       </c>
-      <c r="S98" s="8"/>
+      <c r="S98" s="8" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B99" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A99,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="D99" s="14" t="n">
         <v>1</v>
@@ -6825,14 +6930,14 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B100" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A100,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D100" s="14" t="n">
         <v>0</v>
@@ -6861,19 +6966,19 @@
         <v>0</v>
       </c>
       <c r="S100" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B101" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A101,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D101" s="14" t="n">
         <v>0</v>
@@ -6902,19 +7007,19 @@
         <v>0</v>
       </c>
       <c r="S101" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B102" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A102,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D102" s="14" t="n">
         <v>1</v>
@@ -6943,19 +7048,19 @@
         <v>0</v>
       </c>
       <c r="S102" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B103" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A103,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D103" s="14" t="n">
         <v>1</v>
@@ -6987,14 +7092,14 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B104" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A104,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D104" s="14" t="n">
         <v>1</v>
@@ -7026,14 +7131,14 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B105" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A105,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D105" s="14" t="n">
         <v>0</v>
@@ -7062,19 +7167,19 @@
         <v>0</v>
       </c>
       <c r="S105" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B106" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A106,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D106" s="14" t="n">
         <v>0</v>
@@ -7103,19 +7208,19 @@
         <v>0</v>
       </c>
       <c r="S106" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B107" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A107,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D107" s="14" t="n">
         <v>1</v>
@@ -7144,19 +7249,19 @@
         <v>0</v>
       </c>
       <c r="S107" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B108" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A108,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D108" s="14" t="n">
         <v>1</v>
@@ -7188,14 +7293,14 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B109" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A109,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D109" s="14" t="n">
         <v>1</v>
@@ -7227,14 +7332,14 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B110" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A110,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D110" s="14" t="n">
         <v>0</v>
@@ -7263,19 +7368,19 @@
         <v>0</v>
       </c>
       <c r="S110" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B111" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A111,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D111" s="14" t="n">
         <v>0</v>
@@ -7304,19 +7409,19 @@
         <v>0</v>
       </c>
       <c r="S111" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B112" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A112,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D112" s="14" t="n">
         <v>1</v>
@@ -7345,19 +7450,19 @@
         <v>0</v>
       </c>
       <c r="S112" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B113" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A113,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D113" s="14" t="n">
         <v>1</v>
@@ -7389,14 +7494,14 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B114" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A114,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D114" s="14" t="n">
         <v>1</v>
@@ -7428,14 +7533,14 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B115" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A115,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D115" s="14" t="n">
         <v>0</v>
@@ -7464,19 +7569,19 @@
         <v>0</v>
       </c>
       <c r="S115" s="8" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B116" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A116,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D116" s="14" t="n">
         <v>0</v>
@@ -7505,7 +7610,7 @@
         <v>0</v>
       </c>
       <c r="S116" s="8" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7514,10 +7619,10 @@
       </c>
       <c r="B117" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A117,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D117" s="14" t="n">
         <v>1</v>
@@ -7545,7 +7650,9 @@
         <f aca="false">IF(P117="",0,P117*D117)</f>
         <v>0</v>
       </c>
-      <c r="S117" s="8"/>
+      <c r="S117" s="8" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="6" t="s">
@@ -7553,10 +7660,10 @@
       </c>
       <c r="B118" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A118,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D118" s="14" t="n">
         <v>1</v>
@@ -7584,9 +7691,7 @@
         <f aca="false">IF(P118="",0,P118*D118)</f>
         <v>0</v>
       </c>
-      <c r="S118" s="8" t="s">
-        <v>183</v>
-      </c>
+      <c r="S118" s="8"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="6" t="s">
@@ -7594,13 +7699,13 @@
       </c>
       <c r="B119" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A119,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="D119" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E119" s="14"/>
       <c r="F119" s="14"/>
@@ -7625,9 +7730,7 @@
         <f aca="false">IF(P119="",0,P119*D119)</f>
         <v>0</v>
       </c>
-      <c r="S119" s="8" t="s">
-        <v>178</v>
-      </c>
+      <c r="S119" s="8"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="6" t="s">
@@ -7635,10 +7738,10 @@
       </c>
       <c r="B120" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A120,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D120" s="14" t="n">
         <v>0</v>
@@ -7667,7 +7770,210 @@
         <v>0</v>
       </c>
       <c r="S120" s="8" t="s">
-        <v>180</v>
+        <v>191</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B121" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A121,Киты!$A:$A,0)),"")</f>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+      </c>
+      <c r="C121" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D121" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" s="14"/>
+      <c r="F121" s="14"/>
+      <c r="G121" s="12"/>
+      <c r="H121" s="12"/>
+      <c r="I121" s="12"/>
+      <c r="J121" s="12"/>
+      <c r="K121" s="12"/>
+      <c r="L121" s="12"/>
+      <c r="M121" s="12"/>
+      <c r="N121" s="12"/>
+      <c r="O121" s="12"/>
+      <c r="P121" s="9" t="str">
+        <f aca="false">IF(COUNT(G121:O121)=0,"",MIN(G121:O121))</f>
+        <v/>
+      </c>
+      <c r="Q121" s="7" t="str">
+        <f aca="false">IF(P121="","",INDEX($G$1:$O$1,MATCH(P121,G121:O121,0)))</f>
+        <v/>
+      </c>
+      <c r="R121" s="9" t="n">
+        <f aca="false">IF(P121="",0,P121*D121)</f>
+        <v>0</v>
+      </c>
+      <c r="S121" s="8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B122" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A122,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D122" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E122" s="14"/>
+      <c r="F122" s="14"/>
+      <c r="G122" s="12"/>
+      <c r="H122" s="12"/>
+      <c r="I122" s="12"/>
+      <c r="J122" s="12"/>
+      <c r="K122" s="12"/>
+      <c r="L122" s="12"/>
+      <c r="M122" s="12"/>
+      <c r="N122" s="12"/>
+      <c r="O122" s="12"/>
+      <c r="P122" s="9" t="str">
+        <f aca="false">IF(COUNT(G122:O122)=0,"",MIN(G122:O122))</f>
+        <v/>
+      </c>
+      <c r="Q122" s="7" t="str">
+        <f aca="false">IF(P122="","",INDEX($G$1:$O$1,MATCH(P122,G122:O122,0)))</f>
+        <v/>
+      </c>
+      <c r="R122" s="9" t="n">
+        <f aca="false">IF(P122="",0,P122*D122)</f>
+        <v>0</v>
+      </c>
+      <c r="S122" s="8"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B123" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A123,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D123" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E123" s="14"/>
+      <c r="F123" s="14"/>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+      <c r="I123" s="12"/>
+      <c r="J123" s="12"/>
+      <c r="K123" s="12"/>
+      <c r="L123" s="12"/>
+      <c r="M123" s="12"/>
+      <c r="N123" s="12"/>
+      <c r="O123" s="12"/>
+      <c r="P123" s="9" t="str">
+        <f aca="false">IF(COUNT(G123:O123)=0,"",MIN(G123:O123))</f>
+        <v/>
+      </c>
+      <c r="Q123" s="7" t="str">
+        <f aca="false">IF(P123="","",INDEX($G$1:$O$1,MATCH(P123,G123:O123,0)))</f>
+        <v/>
+      </c>
+      <c r="R123" s="9" t="n">
+        <f aca="false">IF(P123="",0,P123*D123)</f>
+        <v>0</v>
+      </c>
+      <c r="S123" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B124" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A124,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="D124" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" s="14"/>
+      <c r="F124" s="14"/>
+      <c r="G124" s="12"/>
+      <c r="H124" s="12"/>
+      <c r="I124" s="12"/>
+      <c r="J124" s="12"/>
+      <c r="K124" s="12"/>
+      <c r="L124" s="12"/>
+      <c r="M124" s="12"/>
+      <c r="N124" s="12"/>
+      <c r="O124" s="12"/>
+      <c r="P124" s="9" t="str">
+        <f aca="false">IF(COUNT(G124:O124)=0,"",MIN(G124:O124))</f>
+        <v/>
+      </c>
+      <c r="Q124" s="7" t="str">
+        <f aca="false">IF(P124="","",INDEX($G$1:$O$1,MATCH(P124,G124:O124,0)))</f>
+        <v/>
+      </c>
+      <c r="R124" s="9" t="n">
+        <f aca="false">IF(P124="",0,P124*D124)</f>
+        <v>0</v>
+      </c>
+      <c r="S124" s="8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B125" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A125,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D125" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" s="14"/>
+      <c r="F125" s="14"/>
+      <c r="G125" s="12"/>
+      <c r="H125" s="12"/>
+      <c r="I125" s="12"/>
+      <c r="J125" s="12"/>
+      <c r="K125" s="12"/>
+      <c r="L125" s="12"/>
+      <c r="M125" s="12"/>
+      <c r="N125" s="12"/>
+      <c r="O125" s="12"/>
+      <c r="P125" s="9" t="str">
+        <f aca="false">IF(COUNT(G125:O125)=0,"",MIN(G125:O125))</f>
+        <v/>
+      </c>
+      <c r="Q125" s="7" t="str">
+        <f aca="false">IF(P125="","",INDEX($G$1:$O$1,MATCH(P125,G125:O125,0)))</f>
+        <v/>
+      </c>
+      <c r="R125" s="9" t="n">
+        <f aca="false">IF(P125="",0,P125*D125)</f>
+        <v>0</v>
+      </c>
+      <c r="S125" s="8" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -7704,80 +8010,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="E2" s="16" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="I2" s="16" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="J2" s="16" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -7791,10 +8097,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
@@ -7808,10 +8114,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
@@ -7825,10 +8131,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -7842,10 +8148,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -7859,10 +8165,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
@@ -7876,10 +8182,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
@@ -7893,10 +8199,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -7910,10 +8216,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C11" s="22"/>
       <c r="D11" s="22"/>
@@ -7964,7 +8270,7 @@
         <v>14</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>15</v>
@@ -7973,197 +8279,197 @@
         <v>16</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Picanto kit without washer; repair card with brands, QR and A4 sheet
- Picanto TO kit now matches the user's list exactly (washer removed);
  purchase prices stored per item in kits.json
- workbook TO rows are derived from each kit's own contents (no items
  added that the kit does not contain); brands and quoted prices are
  written by the builder
- repair card: skips listing itself, prints known brands with a blank
  article field, draws a QR code when a kit has a "video" link (segno),
  hides the QR block otherwise; A4 sheet with 4 cards for assembled kits
- templates.md: how to print, fill and use the repair card

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="253">
   <si>
     <t xml:space="preserve">ZAPKIT — таблица закупки и цен</t>
   </si>
@@ -595,28 +595,25 @@
     <t xml:space="preserve">Поставьте 1, если объём заливки с фильтром больше 4 л (проверьте по VIN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hyundai/Kia Super Extra Gasoline 5W-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ваша закупка: 2 051,00 ₽ — впишите в колонку поставщика, у которого брали. Проверьте допуск: для Picanto рекомендуют API SM / ILSAC GF-4 и выше.</t>
+    <t xml:space="preserve">Hyundai/Kia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 2 051,00 ₽ — впишите в колонку поставщика, у которого брали. Проверьте допуск: для Picanto рекомендуют API SM / ILSAC GF-4 и выше</t>
   </si>
   <si>
     <t xml:space="preserve">AMD</t>
   </si>
   <si>
-    <t xml:space="preserve">Ваша закупка: 154,70 ₽ — впишите в колонку поставщика, у которого брали.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ваша закупка: 533,00 ₽ — впишите в колонку поставщика, у которого брали.</t>
+    <t xml:space="preserve">Ваша закупка: 154,70 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 533,00 ₽ — впишите в колонку поставщика, у которого брали</t>
   </si>
   <si>
     <t xml:space="preserve">BIG FILTER</t>
   </si>
   <si>
-    <t xml:space="preserve">Ваша закупка: 387,00 ₽ — впишите в колонку поставщика, у которого брали.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Добавлена по стандартному составу ТО-кита; подберите по VIN (обычно 30–60 ₽).</t>
+    <t xml:space="preserve">Ваша закупка: 387,00 ₽ — впишите в колонку поставщика, у которого брали</t>
   </si>
   <si>
     <t xml:space="preserve">Комплект цепи ГРМ (цепь, натяжитель, успокоители)</t>
@@ -2183,7 +2180,7 @@
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A14,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K14" s="11" t="str">
         <f aca="false">IF(I14="","",CEILING(I14*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2934,7 +2931,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S125"/>
+  <dimension ref="A1:S124"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -5845,14 +5842,14 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B73" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A73,Киты!$A:$A,0)),"")</f>
-        <v>Kia Picanto 1.0 / 1.2</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="D73" s="14" t="n">
         <v>1</v>
@@ -5881,7 +5878,7 @@
         <v>0</v>
       </c>
       <c r="S73" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5893,7 +5890,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D74" s="14" t="n">
         <v>1</v>
@@ -5921,9 +5918,7 @@
         <f aca="false">IF(P74="",0,P74*D74)</f>
         <v>0</v>
       </c>
-      <c r="S74" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S74" s="8"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
@@ -5976,7 +5971,7 @@
         <v>189</v>
       </c>
       <c r="D76" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E76" s="14"/>
       <c r="F76" s="14"/>
@@ -6001,7 +5996,9 @@
         <f aca="false">IF(P76="",0,P76*D76)</f>
         <v>0</v>
       </c>
-      <c r="S76" s="8"/>
+      <c r="S76" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
@@ -6012,7 +6009,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D77" s="14" t="n">
         <v>0</v>
@@ -6041,22 +6038,22 @@
         <v>0</v>
       </c>
       <c r="S77" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B78" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A78,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D78" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E78" s="14"/>
       <c r="F78" s="14"/>
@@ -6082,7 +6079,7 @@
         <v>0</v>
       </c>
       <c r="S78" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6094,7 +6091,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D79" s="14" t="n">
         <v>1</v>
@@ -6122,9 +6119,7 @@
         <f aca="false">IF(P79="",0,P79*D79)</f>
         <v>0</v>
       </c>
-      <c r="S79" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S79" s="8"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
@@ -6177,7 +6172,7 @@
         <v>189</v>
       </c>
       <c r="D81" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E81" s="14"/>
       <c r="F81" s="14"/>
@@ -6202,7 +6197,9 @@
         <f aca="false">IF(P81="",0,P81*D81)</f>
         <v>0</v>
       </c>
-      <c r="S81" s="8"/>
+      <c r="S81" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="s">
@@ -6213,7 +6210,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D82" s="14" t="n">
         <v>0</v>
@@ -6242,22 +6239,22 @@
         <v>0</v>
       </c>
       <c r="S82" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B83" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A83,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D83" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E83" s="14"/>
       <c r="F83" s="14"/>
@@ -6283,7 +6280,7 @@
         <v>0</v>
       </c>
       <c r="S83" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6295,7 +6292,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D84" s="14" t="n">
         <v>1</v>
@@ -6323,9 +6320,7 @@
         <f aca="false">IF(P84="",0,P84*D84)</f>
         <v>0</v>
       </c>
-      <c r="S84" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S84" s="8"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="s">
@@ -6378,7 +6373,7 @@
         <v>189</v>
       </c>
       <c r="D86" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E86" s="14"/>
       <c r="F86" s="14"/>
@@ -6403,7 +6398,9 @@
         <f aca="false">IF(P86="",0,P86*D86)</f>
         <v>0</v>
       </c>
-      <c r="S86" s="8"/>
+      <c r="S86" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="6" t="s">
@@ -6414,7 +6411,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D87" s="14" t="n">
         <v>0</v>
@@ -6443,22 +6440,22 @@
         <v>0</v>
       </c>
       <c r="S87" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B88" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A88,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D88" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E88" s="14"/>
       <c r="F88" s="14"/>
@@ -6484,7 +6481,7 @@
         <v>0</v>
       </c>
       <c r="S88" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6496,7 +6493,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D89" s="14" t="n">
         <v>1</v>
@@ -6524,9 +6521,7 @@
         <f aca="false">IF(P89="",0,P89*D89)</f>
         <v>0</v>
       </c>
-      <c r="S89" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S89" s="8"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="6" t="s">
@@ -6579,7 +6574,7 @@
         <v>189</v>
       </c>
       <c r="D91" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E91" s="14"/>
       <c r="F91" s="14"/>
@@ -6604,7 +6599,9 @@
         <f aca="false">IF(P91="",0,P91*D91)</f>
         <v>0</v>
       </c>
-      <c r="S91" s="8"/>
+      <c r="S91" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="6" t="s">
@@ -6615,7 +6612,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D92" s="14" t="n">
         <v>0</v>
@@ -6644,22 +6641,22 @@
         <v>0</v>
       </c>
       <c r="S92" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B93" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A93,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D93" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E93" s="14"/>
       <c r="F93" s="14"/>
@@ -6685,7 +6682,7 @@
         <v>0</v>
       </c>
       <c r="S93" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6697,7 +6694,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D94" s="14" t="n">
         <v>1</v>
@@ -6725,9 +6722,7 @@
         <f aca="false">IF(P94="",0,P94*D94)</f>
         <v>0</v>
       </c>
-      <c r="S94" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S94" s="8"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="6" t="s">
@@ -6780,7 +6775,7 @@
         <v>189</v>
       </c>
       <c r="D96" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E96" s="14"/>
       <c r="F96" s="14"/>
@@ -6805,7 +6800,9 @@
         <f aca="false">IF(P96="",0,P96*D96)</f>
         <v>0</v>
       </c>
-      <c r="S96" s="8"/>
+      <c r="S96" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="6" t="s">
@@ -6816,7 +6813,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D97" s="14" t="n">
         <v>0</v>
@@ -6845,22 +6842,22 @@
         <v>0</v>
       </c>
       <c r="S97" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B98" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A98,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D98" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E98" s="14"/>
       <c r="F98" s="14"/>
@@ -6885,9 +6882,7 @@
         <f aca="false">IF(P98="",0,P98*D98)</f>
         <v>0</v>
       </c>
-      <c r="S98" s="8" t="s">
-        <v>193</v>
-      </c>
+      <c r="S98" s="8"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="6" t="s">
@@ -6898,10 +6893,10 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D99" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E99" s="14"/>
       <c r="F99" s="14"/>
@@ -6926,7 +6921,9 @@
         <f aca="false">IF(P99="",0,P99*D99)</f>
         <v>0</v>
       </c>
-      <c r="S99" s="8"/>
+      <c r="S99" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="6" t="s">
@@ -6937,7 +6934,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D100" s="14" t="n">
         <v>0</v>
@@ -6966,22 +6963,22 @@
         <v>0</v>
       </c>
       <c r="S100" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B101" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A101,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D101" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E101" s="14"/>
       <c r="F101" s="14"/>
@@ -7007,7 +7004,7 @@
         <v>0</v>
       </c>
       <c r="S101" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7019,7 +7016,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D102" s="14" t="n">
         <v>1</v>
@@ -7047,9 +7044,7 @@
         <f aca="false">IF(P102="",0,P102*D102)</f>
         <v>0</v>
       </c>
-      <c r="S102" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S102" s="8"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="6" t="s">
@@ -7102,7 +7097,7 @@
         <v>189</v>
       </c>
       <c r="D104" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E104" s="14"/>
       <c r="F104" s="14"/>
@@ -7127,7 +7122,9 @@
         <f aca="false">IF(P104="",0,P104*D104)</f>
         <v>0</v>
       </c>
-      <c r="S104" s="8"/>
+      <c r="S104" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="6" t="s">
@@ -7138,7 +7135,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D105" s="14" t="n">
         <v>0</v>
@@ -7167,22 +7164,22 @@
         <v>0</v>
       </c>
       <c r="S105" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B106" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A106,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D106" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E106" s="14"/>
       <c r="F106" s="14"/>
@@ -7208,7 +7205,7 @@
         <v>0</v>
       </c>
       <c r="S106" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7220,7 +7217,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D107" s="14" t="n">
         <v>1</v>
@@ -7248,9 +7245,7 @@
         <f aca="false">IF(P107="",0,P107*D107)</f>
         <v>0</v>
       </c>
-      <c r="S107" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S107" s="8"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="6" t="s">
@@ -7303,7 +7298,7 @@
         <v>189</v>
       </c>
       <c r="D109" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E109" s="14"/>
       <c r="F109" s="14"/>
@@ -7328,7 +7323,9 @@
         <f aca="false">IF(P109="",0,P109*D109)</f>
         <v>0</v>
       </c>
-      <c r="S109" s="8"/>
+      <c r="S109" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="6" t="s">
@@ -7339,7 +7336,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D110" s="14" t="n">
         <v>0</v>
@@ -7368,22 +7365,22 @@
         <v>0</v>
       </c>
       <c r="S110" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B111" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A111,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D111" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E111" s="14"/>
       <c r="F111" s="14"/>
@@ -7409,7 +7406,7 @@
         <v>0</v>
       </c>
       <c r="S111" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7421,7 +7418,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D112" s="14" t="n">
         <v>1</v>
@@ -7449,9 +7446,7 @@
         <f aca="false">IF(P112="",0,P112*D112)</f>
         <v>0</v>
       </c>
-      <c r="S112" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S112" s="8"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="6" t="s">
@@ -7504,7 +7499,7 @@
         <v>189</v>
       </c>
       <c r="D114" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E114" s="14"/>
       <c r="F114" s="14"/>
@@ -7529,7 +7524,9 @@
         <f aca="false">IF(P114="",0,P114*D114)</f>
         <v>0</v>
       </c>
-      <c r="S114" s="8"/>
+      <c r="S114" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="6" t="s">
@@ -7540,7 +7537,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D115" s="14" t="n">
         <v>0</v>
@@ -7569,22 +7566,22 @@
         <v>0</v>
       </c>
       <c r="S115" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B116" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A116,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D116" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E116" s="14"/>
       <c r="F116" s="14"/>
@@ -7610,7 +7607,7 @@
         <v>0</v>
       </c>
       <c r="S116" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7622,7 +7619,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D117" s="14" t="n">
         <v>1</v>
@@ -7650,9 +7647,7 @@
         <f aca="false">IF(P117="",0,P117*D117)</f>
         <v>0</v>
       </c>
-      <c r="S117" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="S117" s="8"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="6" t="s">
@@ -7705,7 +7700,7 @@
         <v>189</v>
       </c>
       <c r="D119" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E119" s="14"/>
       <c r="F119" s="14"/>
@@ -7730,7 +7725,9 @@
         <f aca="false">IF(P119="",0,P119*D119)</f>
         <v>0</v>
       </c>
-      <c r="S119" s="8"/>
+      <c r="S119" s="8" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="6" t="s">
@@ -7741,7 +7738,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D120" s="14" t="n">
         <v>0</v>
@@ -7770,22 +7767,22 @@
         <v>0</v>
       </c>
       <c r="S120" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="6" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B121" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A121,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D121" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E121" s="14"/>
       <c r="F121" s="14"/>
@@ -7810,9 +7807,7 @@
         <f aca="false">IF(P121="",0,P121*D121)</f>
         <v>0</v>
       </c>
-      <c r="S121" s="8" t="s">
-        <v>193</v>
-      </c>
+      <c r="S121" s="8"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="6" t="s">
@@ -7851,7 +7846,9 @@
         <f aca="false">IF(P122="",0,P122*D122)</f>
         <v>0</v>
       </c>
-      <c r="S122" s="8"/>
+      <c r="S122" s="8" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="6" t="s">
@@ -7862,10 +7859,10 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D123" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E123" s="14"/>
       <c r="F123" s="14"/>
@@ -7891,7 +7888,7 @@
         <v>0</v>
       </c>
       <c r="S123" s="8" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7903,7 +7900,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D124" s="14" t="n">
         <v>0</v>
@@ -7932,48 +7929,7 @@
         <v>0</v>
       </c>
       <c r="S124" s="8" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B125" s="7" t="str">
-        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A125,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
-      </c>
-      <c r="C125" s="7" t="s">
         <v>192</v>
-      </c>
-      <c r="D125" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E125" s="14"/>
-      <c r="F125" s="14"/>
-      <c r="G125" s="12"/>
-      <c r="H125" s="12"/>
-      <c r="I125" s="12"/>
-      <c r="J125" s="12"/>
-      <c r="K125" s="12"/>
-      <c r="L125" s="12"/>
-      <c r="M125" s="12"/>
-      <c r="N125" s="12"/>
-      <c r="O125" s="12"/>
-      <c r="P125" s="9" t="str">
-        <f aca="false">IF(COUNT(G125:O125)=0,"",MIN(G125:O125))</f>
-        <v/>
-      </c>
-      <c r="Q125" s="7" t="str">
-        <f aca="false">IF(P125="","",INDEX($G$1:$O$1,MATCH(P125,G125:O125,0)))</f>
-        <v/>
-      </c>
-      <c r="R125" s="9" t="n">
-        <f aca="false">IF(P125="",0,P125*D125)</f>
-        <v>0</v>
-      </c>
-      <c r="S125" s="8" t="s">
-        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -8010,34 +7966,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>204</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>205</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>164</v>
@@ -8048,31 +8004,31 @@
         <v>165</v>
       </c>
       <c r="B2" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="C2" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="E2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="E2" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="16" t="s">
+      <c r="G2" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="H2" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="I2" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="J2" s="16" t="s">
         <v>212</v>
-      </c>
-      <c r="J2" s="16" t="s">
-        <v>213</v>
       </c>
       <c r="K2" s="16" t="s">
         <v>166</v>
@@ -8083,7 +8039,7 @@
         <v>152</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -8100,7 +8056,7 @@
         <v>153</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
@@ -8117,7 +8073,7 @@
         <v>154</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
@@ -8134,7 +8090,7 @@
         <v>155</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -8151,7 +8107,7 @@
         <v>156</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -8168,7 +8124,7 @@
         <v>157</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
@@ -8185,7 +8141,7 @@
         <v>158</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
@@ -8202,7 +8158,7 @@
         <v>159</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -8219,7 +8175,7 @@
         <v>160</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C11" s="22"/>
       <c r="D11" s="22"/>
@@ -8270,7 +8226,7 @@
         <v>14</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>15</v>
@@ -8279,197 +8235,197 @@
         <v>16</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>220</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>221</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>223</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>225</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>226</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F3" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>227</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C4" s="8" t="s">
         <v>230</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>231</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>234</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>235</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>238</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>239</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>240</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="8" t="s">
         <v>243</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>244</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>247</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>248</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>250</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>251</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="G9" s="8" t="s">
         <v>252</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add VW Jetta TO kit (TO-14); repair card without QR video for now
- kits.json: TO-14 VW Jetta exactly as assembled (TEBOIL Diamond Multi
  5W-40 4 L, AMD oil filter, BRAVE air and cabin filters) with purchase
  prices; price 5 890 ₽ by the 30% rule
- "Карта ремонта с QR-видео" renamed to "Карта ремонта" on all photos
  and texts; card icon shows a checklist instead of a QR pattern
- listings: per-item listing_name (oil with VW 502 00 / 505 00
  approval), Jetta intro, Jetta in store description
- workbook rebuilt with TO-14 rows; docs counts updated to 25 kits

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="265">
   <si>
     <t xml:space="preserve">ZAPKIT — таблица закупки и цен</t>
   </si>
@@ -349,6 +349,24 @@
     <t xml:space="preserve">to-13-picanto-1-main.png</t>
   </si>
   <si>
+    <t xml:space="preserve">TO-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VW Jetta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">уточнить по VIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТО-кит VW Jetta: масло и фильтры</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to-14-jetta-1-main.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">GRM-01</t>
   </si>
   <si>
@@ -614,6 +632,24 @@
   </si>
   <si>
     <t xml:space="preserve">Ваша закупка: 387,00 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEBOIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 3 525,84 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 308,10 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRAVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 311,00 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 317,00 ₽ — впишите в колонку поставщика, у которого брали</t>
   </si>
   <si>
     <t xml:space="preserve">Комплект цепи ГРМ (цепь, натяжитель, успокоители)</t>
@@ -1430,7 +1466,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -2208,25 +2244,25 @@
         <v>96</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>30</v>
-      </c>
       <c r="D15" s="7" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>33</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I15" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A15)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A15)+Параметры!$B$3)</f>
@@ -2234,7 +2270,7 @@
       </c>
       <c r="J15" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A15,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15" s="11" t="str">
         <f aca="false">IF(I15="","",CEILING(I15*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2259,16 +2295,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>32</v>
@@ -2277,10 +2313,10 @@
         <v>33</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="I16" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A16)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A16)+Параметры!$B$3)</f>
@@ -2313,16 +2349,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>97</v>
-      </c>
       <c r="C17" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>32</v>
@@ -2331,10 +2367,10 @@
         <v>33</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I17" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A17)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A17)+Параметры!$B$3)</f>
@@ -2367,16 +2403,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>32</v>
@@ -2385,10 +2421,10 @@
         <v>33</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="I18" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A18)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A18)+Параметры!$B$3)</f>
@@ -2421,28 +2457,28 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I19" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A19)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A19)+Параметры!$B$3)</f>
@@ -2475,28 +2511,28 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I20" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A20)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A20)+Параметры!$B$3)</f>
@@ -2504,7 +2540,7 @@
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A20,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K20" s="11" t="str">
         <f aca="false">IF(I20="","",CEILING(I20*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2529,28 +2565,28 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="I21" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A21)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A21)+Параметры!$B$3)</f>
@@ -2558,7 +2594,7 @@
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A21,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K21" s="11" t="str">
         <f aca="false">IF(I21="","",CEILING(I21*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2583,28 +2619,28 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I22" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A22)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A22)+Параметры!$B$3)</f>
@@ -2637,28 +2673,28 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="I23" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A23)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A23)+Параметры!$B$3)</f>
@@ -2691,28 +2727,28 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>126</v>
+        <v>72</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I24" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A24)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A24)+Параметры!$B$3)</f>
@@ -2745,28 +2781,28 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>86</v>
+        <v>132</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I25" s="9" t="str">
         <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A25)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A25)+Параметры!$B$3)</f>
@@ -2774,7 +2810,7 @@
       </c>
       <c r="J25" s="10" t="n">
         <f aca="false">COUNTIFS(Состав!$A:$A,A25,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" s="11" t="str">
         <f aca="false">IF(I25="","",CEILING(I25*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
@@ -2797,19 +2833,73 @@
         <v>36</v>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I26" s="9" t="str">
+        <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A26)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A26)+Параметры!$B$3)</f>
+        <v/>
+      </c>
+      <c r="J26" s="10" t="n">
+        <f aca="false">COUNTIFS(Состав!$A:$A,A26,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
+        <v>2</v>
+      </c>
+      <c r="K26" s="11" t="str">
+        <f aca="false">IF(I26="","",CEILING(I26*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)</f>
+        <v/>
+      </c>
+      <c r="L26" s="12"/>
+      <c r="M26" s="7" t="str">
+        <f aca="false">IF(OR(K26="",L26=""),"",IF(K26&lt;=L26,"не дороже рынка","дороже рынка"))</f>
+        <v/>
+      </c>
+      <c r="N26" s="9" t="str">
+        <f aca="false">IF(K26="","",K26-I26-K26*Параметры!$B$6-Параметры!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O26" s="13" t="str">
+        <f aca="false">IF(N26="","",N26/K26)</f>
+        <v/>
+      </c>
+      <c r="P26" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J2:J25">
+  <conditionalFormatting sqref="J2:J26">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M25">
+  <conditionalFormatting sqref="M2:M26">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"дороже рынка"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P25" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P26" type="list">
       <formula1>"не выложен,выложен,есть продажи,снят"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2840,79 +2930,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B2" s="15" t="n">
         <v>0.3</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>50</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>100</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>0.065</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>180</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2931,7 +3021,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S124"/>
+  <dimension ref="A1:S128"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -2955,75 +3045,75 @@
         <v>14</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D2" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="G2" s="19" t="n">
         <v>460</v>
@@ -3055,7 +3145,7 @@
         <v>430</v>
       </c>
       <c r="S2" s="21" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3067,7 +3157,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>1</v>
@@ -3096,7 +3186,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3108,7 +3198,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D4" s="14" t="n">
         <v>1</v>
@@ -3147,7 +3237,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>1</v>
@@ -3186,7 +3276,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>1</v>
@@ -3225,7 +3315,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>1</v>
@@ -3264,7 +3354,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D8" s="14" t="n">
         <v>1</v>
@@ -3293,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3305,7 +3395,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>1</v>
@@ -3344,7 +3434,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>1</v>
@@ -3383,7 +3473,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>1</v>
@@ -3422,7 +3512,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>1</v>
@@ -3461,7 +3551,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>1</v>
@@ -3490,7 +3580,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3502,7 +3592,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D14" s="14" t="n">
         <v>1</v>
@@ -3541,7 +3631,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>1</v>
@@ -3580,7 +3670,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>1</v>
@@ -3619,7 +3709,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>1</v>
@@ -3658,7 +3748,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>1</v>
@@ -3687,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="S18" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3699,7 +3789,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>1</v>
@@ -3738,7 +3828,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D20" s="14" t="n">
         <v>1</v>
@@ -3777,7 +3867,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D21" s="14" t="n">
         <v>1</v>
@@ -3816,7 +3906,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D22" s="14" t="n">
         <v>1</v>
@@ -3855,7 +3945,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D23" s="14" t="n">
         <v>1</v>
@@ -3884,7 +3974,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3896,7 +3986,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D24" s="14" t="n">
         <v>1</v>
@@ -3935,7 +4025,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D25" s="14" t="n">
         <v>1</v>
@@ -3974,7 +4064,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D26" s="14" t="n">
         <v>1</v>
@@ -4013,7 +4103,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D27" s="14" t="n">
         <v>1</v>
@@ -4052,7 +4142,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D28" s="14" t="n">
         <v>1</v>
@@ -4081,7 +4171,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4093,7 +4183,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D29" s="14" t="n">
         <v>1</v>
@@ -4132,7 +4222,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D30" s="14" t="n">
         <v>1</v>
@@ -4171,7 +4261,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D31" s="14" t="n">
         <v>1</v>
@@ -4210,7 +4300,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D32" s="14" t="n">
         <v>1</v>
@@ -4249,7 +4339,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D33" s="14" t="n">
         <v>1</v>
@@ -4278,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="S33" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4290,7 +4380,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D34" s="14" t="n">
         <v>0</v>
@@ -4319,7 +4409,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4331,7 +4421,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D35" s="14" t="n">
         <v>1</v>
@@ -4370,7 +4460,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>1</v>
@@ -4409,7 +4499,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D37" s="14" t="n">
         <v>1</v>
@@ -4448,7 +4538,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D38" s="14" t="n">
         <v>1</v>
@@ -4487,7 +4577,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D39" s="14" t="n">
         <v>1</v>
@@ -4516,7 +4606,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4528,7 +4618,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>0</v>
@@ -4557,7 +4647,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4569,7 +4659,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D41" s="14" t="n">
         <v>1</v>
@@ -4608,7 +4698,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D42" s="14" t="n">
         <v>1</v>
@@ -4647,7 +4737,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D43" s="14" t="n">
         <v>1</v>
@@ -4686,7 +4776,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D44" s="14" t="n">
         <v>1</v>
@@ -4725,7 +4815,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D45" s="14" t="n">
         <v>1</v>
@@ -4754,7 +4844,7 @@
         <v>0</v>
       </c>
       <c r="S45" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4766,7 +4856,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D46" s="14" t="n">
         <v>0</v>
@@ -4795,7 +4885,7 @@
         <v>0</v>
       </c>
       <c r="S46" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4807,7 +4897,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D47" s="14" t="n">
         <v>1</v>
@@ -4846,7 +4936,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D48" s="14" t="n">
         <v>1</v>
@@ -4885,7 +4975,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D49" s="14" t="n">
         <v>1</v>
@@ -4924,7 +5014,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D50" s="14" t="n">
         <v>1</v>
@@ -4963,7 +5053,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D51" s="14" t="n">
         <v>1</v>
@@ -4992,7 +5082,7 @@
         <v>0</v>
       </c>
       <c r="S51" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5004,7 +5094,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D52" s="14" t="n">
         <v>0</v>
@@ -5033,7 +5123,7 @@
         <v>0</v>
       </c>
       <c r="S52" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5045,7 +5135,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D53" s="14" t="n">
         <v>1</v>
@@ -5084,7 +5174,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D54" s="14" t="n">
         <v>1</v>
@@ -5123,7 +5213,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D55" s="14" t="n">
         <v>1</v>
@@ -5162,7 +5252,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D56" s="14" t="n">
         <v>1</v>
@@ -5201,7 +5291,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D57" s="14" t="n">
         <v>1</v>
@@ -5230,7 +5320,7 @@
         <v>0</v>
       </c>
       <c r="S57" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5242,7 +5332,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D58" s="14" t="n">
         <v>0</v>
@@ -5271,7 +5361,7 @@
         <v>0</v>
       </c>
       <c r="S58" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5283,7 +5373,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D59" s="14" t="n">
         <v>1</v>
@@ -5322,7 +5412,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D60" s="14" t="n">
         <v>1</v>
@@ -5361,7 +5451,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D61" s="14" t="n">
         <v>1</v>
@@ -5400,7 +5490,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D62" s="14" t="n">
         <v>1</v>
@@ -5439,7 +5529,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D63" s="14" t="n">
         <v>1</v>
@@ -5468,7 +5558,7 @@
         <v>0</v>
       </c>
       <c r="S63" s="8" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5480,7 +5570,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D64" s="14" t="n">
         <v>0</v>
@@ -5509,7 +5599,7 @@
         <v>0</v>
       </c>
       <c r="S64" s="8" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5521,7 +5611,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D65" s="14" t="n">
         <v>1</v>
@@ -5560,7 +5650,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D66" s="14" t="n">
         <v>1</v>
@@ -5599,7 +5689,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D67" s="14" t="n">
         <v>1</v>
@@ -5638,7 +5728,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D68" s="14" t="n">
         <v>1</v>
@@ -5677,13 +5767,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D69" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F69" s="14"/>
       <c r="G69" s="12"/>
@@ -5708,7 +5798,7 @@
         <v>0</v>
       </c>
       <c r="S69" s="8" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5720,13 +5810,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D70" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="F70" s="14"/>
       <c r="G70" s="12"/>
@@ -5751,7 +5841,7 @@
         <v>0</v>
       </c>
       <c r="S70" s="8" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5763,13 +5853,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D71" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E71" s="14" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="F71" s="14"/>
       <c r="G71" s="12"/>
@@ -5794,7 +5884,7 @@
         <v>0</v>
       </c>
       <c r="S71" s="8" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5806,13 +5896,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D72" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F72" s="14"/>
       <c r="G72" s="12"/>
@@ -5837,7 +5927,7 @@
         <v>0</v>
       </c>
       <c r="S72" s="8" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5846,15 +5936,17 @@
       </c>
       <c r="B73" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A73,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>VW Jetta</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D73" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E73" s="14"/>
+      <c r="E73" s="14" t="s">
+        <v>191</v>
+      </c>
       <c r="F73" s="14"/>
       <c r="G73" s="12"/>
       <c r="H73" s="12"/>
@@ -5878,7 +5970,7 @@
         <v>0</v>
       </c>
       <c r="S73" s="8" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5887,15 +5979,17 @@
       </c>
       <c r="B74" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A74,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>VW Jetta</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="D74" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E74" s="14"/>
+      <c r="E74" s="14" t="s">
+        <v>186</v>
+      </c>
       <c r="F74" s="14"/>
       <c r="G74" s="12"/>
       <c r="H74" s="12"/>
@@ -5918,7 +6012,9 @@
         <f aca="false">IF(P74="",0,P74*D74)</f>
         <v>0</v>
       </c>
-      <c r="S74" s="8"/>
+      <c r="S74" s="8" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
@@ -5926,15 +6022,17 @@
       </c>
       <c r="B75" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A75,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>VW Jetta</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D75" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E75" s="14"/>
+      <c r="E75" s="14" t="s">
+        <v>194</v>
+      </c>
       <c r="F75" s="14"/>
       <c r="G75" s="12"/>
       <c r="H75" s="12"/>
@@ -5957,7 +6055,9 @@
         <f aca="false">IF(P75="",0,P75*D75)</f>
         <v>0</v>
       </c>
-      <c r="S75" s="8"/>
+      <c r="S75" s="8" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
@@ -5965,15 +6065,17 @@
       </c>
       <c r="B76" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A76,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2010–2017</v>
+        <v>VW Jetta</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="D76" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E76" s="14"/>
+        <v>1</v>
+      </c>
+      <c r="E76" s="14" t="s">
+        <v>194</v>
+      </c>
       <c r="F76" s="14"/>
       <c r="G76" s="12"/>
       <c r="H76" s="12"/>
@@ -5997,22 +6099,22 @@
         <v>0</v>
       </c>
       <c r="S76" s="8" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B77" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A77,Киты!$A:$A,0)),"")</f>
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D77" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E77" s="14"/>
       <c r="F77" s="14"/>
@@ -6038,19 +6140,19 @@
         <v>0</v>
       </c>
       <c r="S77" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B78" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A78,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D78" s="14" t="n">
         <v>1</v>
@@ -6078,20 +6180,18 @@
         <f aca="false">IF(P78="",0,P78*D78)</f>
         <v>0</v>
       </c>
-      <c r="S78" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S78" s="8"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B79" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A79,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D79" s="14" t="n">
         <v>1</v>
@@ -6123,17 +6223,17 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B80" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A80,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D80" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E80" s="14"/>
       <c r="F80" s="14"/>
@@ -6158,18 +6258,20 @@
         <f aca="false">IF(P80="",0,P80*D80)</f>
         <v>0</v>
       </c>
-      <c r="S80" s="8"/>
+      <c r="S80" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B81" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A81,Киты!$A:$A,0)),"")</f>
-        <v>Hyundai Solaris 2017–2022</v>
+        <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D81" s="14" t="n">
         <v>0</v>
@@ -6198,22 +6300,22 @@
         <v>0</v>
       </c>
       <c r="S81" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B82" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A82,Киты!$A:$A,0)),"")</f>
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D82" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E82" s="14"/>
       <c r="F82" s="14"/>
@@ -6239,19 +6341,19 @@
         <v>0</v>
       </c>
       <c r="S82" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B83" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A83,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D83" s="14" t="n">
         <v>1</v>
@@ -6279,20 +6381,18 @@
         <f aca="false">IF(P83="",0,P83*D83)</f>
         <v>0</v>
       </c>
-      <c r="S83" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S83" s="8"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B84" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A84,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D84" s="14" t="n">
         <v>1</v>
@@ -6324,17 +6424,17 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B85" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A85,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D85" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E85" s="14"/>
       <c r="F85" s="14"/>
@@ -6359,18 +6459,20 @@
         <f aca="false">IF(P85="",0,P85*D85)</f>
         <v>0</v>
       </c>
-      <c r="S85" s="8"/>
+      <c r="S85" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B86" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A86,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2011–2017</v>
+        <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D86" s="14" t="n">
         <v>0</v>
@@ -6399,22 +6501,22 @@
         <v>0</v>
       </c>
       <c r="S86" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="6" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B87" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A87,Киты!$A:$A,0)),"")</f>
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D87" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E87" s="14"/>
       <c r="F87" s="14"/>
@@ -6440,19 +6542,19 @@
         <v>0</v>
       </c>
       <c r="S87" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B88" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A88,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D88" s="14" t="n">
         <v>1</v>
@@ -6480,20 +6582,18 @@
         <f aca="false">IF(P88="",0,P88*D88)</f>
         <v>0</v>
       </c>
-      <c r="S88" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S88" s="8"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B89" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A89,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D89" s="14" t="n">
         <v>1</v>
@@ -6525,17 +6625,17 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B90" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A90,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D90" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E90" s="14"/>
       <c r="F90" s="14"/>
@@ -6560,18 +6660,20 @@
         <f aca="false">IF(P90="",0,P90*D90)</f>
         <v>0</v>
       </c>
-      <c r="S90" s="8"/>
+      <c r="S90" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B91" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A91,Киты!$A:$A,0)),"")</f>
-        <v>Kia Rio 2017–2021</v>
+        <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D91" s="14" t="n">
         <v>0</v>
@@ -6600,22 +6702,22 @@
         <v>0</v>
       </c>
       <c r="S91" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="6" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B92" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A92,Киты!$A:$A,0)),"")</f>
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D92" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E92" s="14"/>
       <c r="F92" s="14"/>
@@ -6641,19 +6743,19 @@
         <v>0</v>
       </c>
       <c r="S92" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B93" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A93,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D93" s="14" t="n">
         <v>1</v>
@@ -6681,20 +6783,18 @@
         <f aca="false">IF(P93="",0,P93*D93)</f>
         <v>0</v>
       </c>
-      <c r="S93" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S93" s="8"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B94" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A94,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D94" s="14" t="n">
         <v>1</v>
@@ -6726,17 +6826,17 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B95" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A95,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D95" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E95" s="14"/>
       <c r="F95" s="14"/>
@@ -6761,18 +6861,20 @@
         <f aca="false">IF(P95="",0,P95*D95)</f>
         <v>0</v>
       </c>
-      <c r="S95" s="8"/>
+      <c r="S95" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B96" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A96,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CFNA</v>
+        <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D96" s="14" t="n">
         <v>0</v>
@@ -6801,22 +6903,22 @@
         <v>0</v>
       </c>
       <c r="S96" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B97" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A97,Киты!$A:$A,0)),"")</f>
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D97" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E97" s="14"/>
       <c r="F97" s="14"/>
@@ -6842,19 +6944,19 @@
         <v>0</v>
       </c>
       <c r="S97" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B98" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A98,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D98" s="14" t="n">
         <v>1</v>
@@ -6886,17 +6988,17 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B99" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A99,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="D99" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E99" s="14"/>
       <c r="F99" s="14"/>
@@ -6921,20 +7023,18 @@
         <f aca="false">IF(P99="",0,P99*D99)</f>
         <v>0</v>
       </c>
-      <c r="S99" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="S99" s="8"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B100" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A100,Киты!$A:$A,0)),"")</f>
-        <v>VW Polo 1.6 CWVA</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="D100" s="14" t="n">
         <v>0</v>
@@ -6963,22 +7063,22 @@
         <v>0</v>
       </c>
       <c r="S100" s="8" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B101" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A101,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
       <c r="D101" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E101" s="14"/>
       <c r="F101" s="14"/>
@@ -7004,19 +7104,19 @@
         <v>0</v>
       </c>
       <c r="S101" s="8" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B102" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A102,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="D102" s="14" t="n">
         <v>1</v>
@@ -7048,17 +7148,17 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B103" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A103,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D103" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" s="14"/>
       <c r="F103" s="14"/>
@@ -7083,18 +7183,20 @@
         <f aca="false">IF(P103="",0,P103*D103)</f>
         <v>0</v>
       </c>
-      <c r="S103" s="8"/>
+      <c r="S103" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B104" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A104,Киты!$A:$A,0)),"")</f>
-        <v>Haval Jolion 1.5T</v>
+        <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D104" s="14" t="n">
         <v>0</v>
@@ -7123,22 +7225,22 @@
         <v>0</v>
       </c>
       <c r="S104" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B105" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A105,Киты!$A:$A,0)),"")</f>
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D105" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" s="14"/>
       <c r="F105" s="14"/>
@@ -7164,19 +7266,19 @@
         <v>0</v>
       </c>
       <c r="S105" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B106" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A106,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D106" s="14" t="n">
         <v>1</v>
@@ -7204,20 +7306,18 @@
         <f aca="false">IF(P106="",0,P106*D106)</f>
         <v>0</v>
       </c>
-      <c r="S106" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S106" s="8"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B107" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A107,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D107" s="14" t="n">
         <v>1</v>
@@ -7249,17 +7349,17 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B108" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A108,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D108" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E108" s="14"/>
       <c r="F108" s="14"/>
@@ -7284,18 +7384,20 @@
         <f aca="false">IF(P108="",0,P108*D108)</f>
         <v>0</v>
       </c>
-      <c r="S108" s="8"/>
+      <c r="S108" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B109" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A109,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 1.5T</v>
+        <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D109" s="14" t="n">
         <v>0</v>
@@ -7324,22 +7426,22 @@
         <v>0</v>
       </c>
       <c r="S109" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B110" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A110,Киты!$A:$A,0)),"")</f>
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D110" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E110" s="14"/>
       <c r="F110" s="14"/>
@@ -7365,19 +7467,19 @@
         <v>0</v>
       </c>
       <c r="S110" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B111" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A111,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D111" s="14" t="n">
         <v>1</v>
@@ -7405,20 +7507,18 @@
         <f aca="false">IF(P111="",0,P111*D111)</f>
         <v>0</v>
       </c>
-      <c r="S111" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S111" s="8"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B112" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A112,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D112" s="14" t="n">
         <v>1</v>
@@ -7450,17 +7550,17 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B113" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A113,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D113" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E113" s="14"/>
       <c r="F113" s="14"/>
@@ -7485,18 +7585,20 @@
         <f aca="false">IF(P113="",0,P113*D113)</f>
         <v>0</v>
       </c>
-      <c r="S113" s="8"/>
+      <c r="S113" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B114" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A114,Киты!$A:$A,0)),"")</f>
-        <v>Haval F7 / F7x 2.0T</v>
+        <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D114" s="14" t="n">
         <v>0</v>
@@ -7525,22 +7627,22 @@
         <v>0</v>
       </c>
       <c r="S114" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B115" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A115,Киты!$A:$A,0)),"")</f>
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D115" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E115" s="14"/>
       <c r="F115" s="14"/>
@@ -7566,19 +7668,19 @@
         <v>0</v>
       </c>
       <c r="S115" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B116" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A116,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="D116" s="14" t="n">
         <v>1</v>
@@ -7606,20 +7708,18 @@
         <f aca="false">IF(P116="",0,P116*D116)</f>
         <v>0</v>
       </c>
-      <c r="S116" s="8" t="s">
-        <v>186</v>
-      </c>
+      <c r="S116" s="8"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B117" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A117,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D117" s="14" t="n">
         <v>1</v>
@@ -7651,17 +7751,17 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B118" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A118,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D118" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E118" s="14"/>
       <c r="F118" s="14"/>
@@ -7686,18 +7786,20 @@
         <f aca="false">IF(P118="",0,P118*D118)</f>
         <v>0</v>
       </c>
-      <c r="S118" s="8"/>
+      <c r="S118" s="8" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B119" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A119,Киты!$A:$A,0)),"")</f>
-        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
+        <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D119" s="14" t="n">
         <v>0</v>
@@ -7726,22 +7828,22 @@
         <v>0</v>
       </c>
       <c r="S119" s="8" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B120" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A120,Киты!$A:$A,0)),"")</f>
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D120" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E120" s="14"/>
       <c r="F120" s="14"/>
@@ -7767,19 +7869,19 @@
         <v>0</v>
       </c>
       <c r="S120" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B121" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A121,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D121" s="14" t="n">
         <v>1</v>
@@ -7811,14 +7913,14 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B122" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A122,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D122" s="14" t="n">
         <v>1</v>
@@ -7846,20 +7948,18 @@
         <f aca="false">IF(P122="",0,P122*D122)</f>
         <v>0</v>
       </c>
-      <c r="S122" s="8" t="s">
-        <v>195</v>
-      </c>
+      <c r="S122" s="8"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B123" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A123,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="D123" s="14" t="n">
         <v>0</v>
@@ -7888,19 +7988,19 @@
         <v>0</v>
       </c>
       <c r="S123" s="8" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B124" s="7" t="str">
         <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A124,Киты!$A:$A,0)),"")</f>
-        <v>Geely Coolray 1.5T</v>
+        <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="D124" s="14" t="n">
         <v>0</v>
@@ -7929,7 +8029,169 @@
         <v>0</v>
       </c>
       <c r="S124" s="8" t="s">
-        <v>192</v>
+        <v>204</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B125" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A125,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D125" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E125" s="14"/>
+      <c r="F125" s="14"/>
+      <c r="G125" s="12"/>
+      <c r="H125" s="12"/>
+      <c r="I125" s="12"/>
+      <c r="J125" s="12"/>
+      <c r="K125" s="12"/>
+      <c r="L125" s="12"/>
+      <c r="M125" s="12"/>
+      <c r="N125" s="12"/>
+      <c r="O125" s="12"/>
+      <c r="P125" s="9" t="str">
+        <f aca="false">IF(COUNT(G125:O125)=0,"",MIN(G125:O125))</f>
+        <v/>
+      </c>
+      <c r="Q125" s="7" t="str">
+        <f aca="false">IF(P125="","",INDEX($G$1:$O$1,MATCH(P125,G125:O125,0)))</f>
+        <v/>
+      </c>
+      <c r="R125" s="9" t="n">
+        <f aca="false">IF(P125="",0,P125*D125)</f>
+        <v>0</v>
+      </c>
+      <c r="S125" s="8"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B126" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A126,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="D126" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E126" s="14"/>
+      <c r="F126" s="14"/>
+      <c r="G126" s="12"/>
+      <c r="H126" s="12"/>
+      <c r="I126" s="12"/>
+      <c r="J126" s="12"/>
+      <c r="K126" s="12"/>
+      <c r="L126" s="12"/>
+      <c r="M126" s="12"/>
+      <c r="N126" s="12"/>
+      <c r="O126" s="12"/>
+      <c r="P126" s="9" t="str">
+        <f aca="false">IF(COUNT(G126:O126)=0,"",MIN(G126:O126))</f>
+        <v/>
+      </c>
+      <c r="Q126" s="7" t="str">
+        <f aca="false">IF(P126="","",INDEX($G$1:$O$1,MATCH(P126,G126:O126,0)))</f>
+        <v/>
+      </c>
+      <c r="R126" s="9" t="n">
+        <f aca="false">IF(P126="",0,P126*D126)</f>
+        <v>0</v>
+      </c>
+      <c r="S126" s="8" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B127" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A127,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C127" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D127" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" s="14"/>
+      <c r="F127" s="14"/>
+      <c r="G127" s="12"/>
+      <c r="H127" s="12"/>
+      <c r="I127" s="12"/>
+      <c r="J127" s="12"/>
+      <c r="K127" s="12"/>
+      <c r="L127" s="12"/>
+      <c r="M127" s="12"/>
+      <c r="N127" s="12"/>
+      <c r="O127" s="12"/>
+      <c r="P127" s="9" t="str">
+        <f aca="false">IF(COUNT(G127:O127)=0,"",MIN(G127:O127))</f>
+        <v/>
+      </c>
+      <c r="Q127" s="7" t="str">
+        <f aca="false">IF(P127="","",INDEX($G$1:$O$1,MATCH(P127,G127:O127,0)))</f>
+        <v/>
+      </c>
+      <c r="R127" s="9" t="n">
+        <f aca="false">IF(P127="",0,P127*D127)</f>
+        <v>0</v>
+      </c>
+      <c r="S127" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B128" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A128,Киты!$A:$A,0)),"")</f>
+        <v>Geely Coolray 1.5T</v>
+      </c>
+      <c r="C128" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D128" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" s="14"/>
+      <c r="F128" s="14"/>
+      <c r="G128" s="12"/>
+      <c r="H128" s="12"/>
+      <c r="I128" s="12"/>
+      <c r="J128" s="12"/>
+      <c r="K128" s="12"/>
+      <c r="L128" s="12"/>
+      <c r="M128" s="12"/>
+      <c r="N128" s="12"/>
+      <c r="O128" s="12"/>
+      <c r="P128" s="9" t="str">
+        <f aca="false">IF(COUNT(G128:O128)=0,"",MIN(G128:O128))</f>
+        <v/>
+      </c>
+      <c r="Q128" s="7" t="str">
+        <f aca="false">IF(P128="","",INDEX($G$1:$O$1,MATCH(P128,G128:O128,0)))</f>
+        <v/>
+      </c>
+      <c r="R128" s="9" t="n">
+        <f aca="false">IF(P128="",0,P128*D128)</f>
+        <v>0</v>
+      </c>
+      <c r="S128" s="8" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -7966,80 +8228,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="E2" s="16" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="I2" s="16" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="J2" s="16" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -8053,10 +8315,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
@@ -8070,10 +8332,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
@@ -8087,10 +8349,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -8104,10 +8366,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -8121,10 +8383,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
@@ -8138,10 +8400,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
@@ -8155,10 +8417,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -8172,10 +8434,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C11" s="22"/>
       <c r="D11" s="22"/>
@@ -8226,7 +8488,7 @@
         <v>14</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>15</v>
@@ -8235,197 +8497,197 @@
         <v>16</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>239</v>
-      </c>
       <c r="G9" s="8" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Coolray GRM kit: XIBTK007 (belt + 2 rollers) and pump belt, price 12 590 ₽
- GRM-12 assembled from real purchase prices: XIAOLU XIBTK007 8 582 ₽,
  pump drive belt 990,23 ₽; no alternator belt (not in the schedule)
- Rollers shown as part of the XIBTK007 set, 3-day lead note in the listing
- Repair cards print the known article; A4 sheet for the priced kit
- Workbook: assembled GRM kits list their real items, article column filled

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="323">
   <si>
     <t xml:space="preserve">ZAPKIT — таблица закупки и цен</t>
   </si>
@@ -515,7 +515,7 @@
     <t xml:space="preserve">GRM-12</t>
   </si>
   <si>
-    <t xml:space="preserve">ГРМ-кит Geely Coolray 1.5T: 2 ремня и ролик</t>
+    <t xml:space="preserve">ГРМ-кит Geely Coolray 1.5T: 2 ремня и 2 ролика</t>
   </si>
   <si>
     <t xml:space="preserve">grm-12-coolray-1-main.png</t>
@@ -854,10 +854,22 @@
     <t xml:space="preserve">Комплект ремня ГРМ (ремень, натяжной ролик)</t>
   </si>
   <si>
+    <t xml:space="preserve">Комплект ГРМ XIAOLU XIBTK007: ремень и 2 ролика</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XIAOLU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XIBTK007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 8 582,00 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ремень привода помпы</t>
   </si>
   <si>
-    <t xml:space="preserve">По регламенту меняется вместе с ремнём ГРМ</t>
+    <t xml:space="preserve">Ваша закупка: 990,23 ₽ — впишите в колонку поставщика, у которого брали</t>
   </si>
   <si>
     <t xml:space="preserve">Поставщик</t>
@@ -9646,13 +9658,17 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C125" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D125" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E125" s="14"/>
-      <c r="F125" s="14"/>
+      <c r="E125" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="F125" s="14" t="s">
+        <v>262</v>
+      </c>
       <c r="G125" s="12"/>
       <c r="H125" s="12"/>
       <c r="I125" s="12"/>
@@ -9674,7 +9690,9 @@
         <f aca="false">IF(P125="",0,P125*D125)</f>
         <v>0</v>
       </c>
-      <c r="S125" s="8"/>
+      <c r="S125" s="8" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="6" t="s">
@@ -9685,7 +9703,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C126" s="7" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D126" s="14" t="n">
         <v>1</v>
@@ -9714,7 +9732,7 @@
         <v>0</v>
       </c>
       <c r="S126" s="8" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9833,34 +9851,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>37</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>224</v>
@@ -9871,31 +9889,31 @@
         <v>225</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E2" s="20" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="K2" s="20" t="s">
         <v>226</v>
@@ -9906,7 +9924,7 @@
         <v>212</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -9923,7 +9941,7 @@
         <v>213</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
@@ -9940,7 +9958,7 @@
         <v>214</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
@@ -9957,7 +9975,7 @@
         <v>215</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -9974,7 +9992,7 @@
         <v>216</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
@@ -9991,7 +10009,7 @@
         <v>217</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
@@ -10008,7 +10026,7 @@
         <v>218</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
@@ -10025,7 +10043,7 @@
         <v>219</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -10042,7 +10060,7 @@
         <v>220</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -10093,7 +10111,7 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>17</v>
@@ -10102,197 +10120,197 @@
         <v>18</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F4" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>297</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>68</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>297</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>98</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Workbook: monthly forecast split into TO and GRM kits
- Separate average check and parts cost for TO (4 490 / 3 365) and
  GRM (Coolray on Gates: 9 990 / 7 056,23), shared Avito share
- Per-order profit and break-even for each kit type
- Scenario table: GRM only (5–30 per month), TO only, TO + GRM mixes
- Reference averages per kit type from the «Киты» sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="333">
   <si>
     <t xml:space="preserve">ZAPKIT — таблица закупки и цен</t>
   </si>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">4. «Параметры» — наценка, комиссии, резерв на товар, постоянные расходы и план заказов. Поменяете там — пересчитается всё.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. «Прогноз» — выручка и прибыль за месяц при разном числе заказов, точка безубыточности.</t>
+    <t xml:space="preserve">5. «Прогноз» — выручка и прибыль за месяц: ТО-киты и ГРМ-киты отдельно и вместе, точка безубыточности.</t>
   </si>
   <si>
     <t xml:space="preserve">6. «Моторы» — справка: где цепь, где ремень, что входит в ГРМ-кит, источники.</t>
@@ -560,25 +560,34 @@
     <t xml:space="preserve">grm-12-coolray-1-main.png</t>
   </si>
   <si>
-    <t xml:space="preserve">Прогноз на месяц (до налога)</t>
+    <t xml:space="preserve">Прогноз на месяц (до налога): ТО-киты и ГРМ-киты</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТО-кит</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ГРМ-кит</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пояснение</t>
   </si>
   <si>
     <t xml:space="preserve">Средний чек кита, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Среднее по собранным китам Picanto (4 190) и Jetta (4 790). Замените, когда соберёте больше китов.</t>
+    <t xml:space="preserve">ТО: среднее по Picanto (4 190) и Jetta (4 790). ГРМ: пока собран один — Coolray на Gates (9 990). Когда соберёте больше китов, возьмите средние из справки ниже.</t>
   </si>
   <si>
     <t xml:space="preserve">Средняя стоимость деталей, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Среднее по Picanto (3 126) и Jetta (3 604).</t>
+    <t xml:space="preserve">ТО: среднее по Picanto и Jetta. ГРМ: Coolray — Gates K0120529 6 066 + ремень помпы 990,23.</t>
   </si>
   <si>
     <t xml:space="preserve">Доля оплат через Авито Доставку</t>
   </si>
   <si>
-    <t xml:space="preserve">Остальные — прямым переводом. Ваша оценка; уточните по факту.</t>
+    <t xml:space="preserve">Общая для ТО и ГРМ. Остальные — прямым переводом. Ваша оценка; уточните по факту.</t>
   </si>
   <si>
     <t xml:space="preserve">Справка: средний чек по листу «Киты»</t>
@@ -590,7 +599,7 @@
     <t xml:space="preserve">Постоянные расходы в месяц, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Сумма постоянных расходов с листа «Параметры».</t>
+    <t xml:space="preserve">Сумма постоянных расходов с листа «Параметры». Платятся один раз в месяц на весь магазин.</t>
   </si>
   <si>
     <t xml:space="preserve">Прибыль с 1 заказа до постоянных расходов, ₽</t>
@@ -599,7 +608,16 @@
     <t xml:space="preserve">Точка безубыточности, заказов в месяц</t>
   </si>
   <si>
-    <t xml:space="preserve">Заказов в месяц</t>
+    <t xml:space="preserve">Сколько китов одного вида нужно продать, чтобы покрыть постоянные расходы.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сценарий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТО-китов в месяц</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ГРМ-китов в месяц</t>
   </si>
   <si>
     <t xml:space="preserve">Выручка, ₽</t>
@@ -620,7 +638,16 @@
     <t xml:space="preserve">Прибыль на 1 заказ, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Налог не учтён. Число заказов в колонке A можно менять. При росте продаж впишите в «Параметры» подписку Авито Pro, если подключите.</t>
+    <t xml:space="preserve">Только ГРМ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Только ТО — для сравнения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТО + ГРМ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Налог не учтён. Число китов в колонках B и C можно менять. При росте продаж впишите в «Параметры» подписку Авито Pro, если подключите.</t>
   </si>
   <si>
     <t xml:space="preserve">Параметр</t>
@@ -4061,16 +4088,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4078,388 +4105,738 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="C3" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="12" t="n">
         <v>4490</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="B4" s="12" t="n">
-        <v>3365</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="D4" s="8"/>
+      <c r="C4" s="12" t="n">
+        <v>9990</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>155</v>
+      </c>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B5" s="15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C5" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="D5" s="8"/>
+      <c r="B5" s="12" t="n">
+        <v>3365</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>7056.23</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>157</v>
+      </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="B6" s="9" t="str">
-        <f aca="false">IFERROR(AVERAGEIF(Киты!$M:$M,"&gt;0"),"")</f>
-        <v/>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B7" s="9" t="str">
-        <f aca="false">IFERROR(AVERAGEIF(Киты!$I:$I,"&gt;0"),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <f aca="false">IFERROR(AVERAGEIFS(Киты!$M:$M,Киты!$B:$B,"ТО",Киты!$M:$M,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="C7" s="9" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Киты!$M:$M,Киты!$B:$B,"ГРМ",Киты!$M:$M,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="B8" s="9" t="n">
+        <v>161</v>
+      </c>
+      <c r="B8" s="9" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Киты!$I:$I,Киты!$B:$B,"ТО",Киты!$I:$I,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="C8" s="9" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Киты!$I:$I,Киты!$B:$B,"ГРМ",Киты!$I:$I,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="9" t="n">
         <f aca="false">(Параметры!$B$12+Параметры!$B$13+Параметры!$B$14+Параметры!$B$15+Параметры!$B$16)</f>
         <v>6783</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="B9" s="9" t="n">
-        <f aca="false">B3-(B4+Параметры!$B$3)-B5*B3*Параметры!$B$6-(1-B5)*(B3*Параметры!$B$10+Параметры!$B$11)-Параметры!$B$7-B4*Параметры!$B$8</f>
+      <c r="D9" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <f aca="false">B4-(B5+Параметры!$B$3)-$B$6*B4*Параметры!$B$6-(1-$B$6)*(B4*Параметры!$B$10+Параметры!$B$11)-Параметры!$B$7-B5*Параметры!$B$8</f>
         <v>565.11</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="B10" s="6" t="n">
-        <f aca="false">IF(B9&lt;=0,"не окупается",ROUNDUP(B8/B9,0))</f>
+      <c r="C10" s="11" t="n">
+        <f aca="false">C4-(C5+Параметры!$B$3)-$B$6*C4*Параметры!$B$6-(1-$B$6)*(C4*Параметры!$B$10+Параметры!$B$11)-Параметры!$B$7-C5*Параметры!$B$8</f>
+        <v>1991.3185</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <f aca="false">IF(B10&lt;=0,"не окупается",ROUNDUP($B$9/B10,0))</f>
         <v>13</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="C11" s="6" t="n">
+        <f aca="false">IF(C10&lt;=0,"не окупается",ROUNDUP($B$9/C10,0))</f>
+        <v>4</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="n">
+      <c r="J13" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <f aca="false">B14*$B$4+C14*$C$4</f>
+        <v>49950</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <f aca="false">B14*($B$5+Параметры!$B$3)+C14*($C$5+Параметры!$B$3)</f>
+        <v>35531.15</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <f aca="false">$B$6*D14*Параметры!$B$6</f>
+        <v>1623.375</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <f aca="false">(1-$B$6)*D14*Параметры!$B$10</f>
+        <v>174.825</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <f aca="false">(B14+C14)*Параметры!$B$7</f>
+        <v>900</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <f aca="false">(B14*$B$5+C14*$C$5)*Параметры!$B$8</f>
+        <v>1764.0575</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <f aca="false">(B14+C14)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <f aca="false">$B$9</f>
+        <v>6783</v>
+      </c>
+      <c r="L14" s="11" t="n">
+        <f aca="false">D14-SUM(E14:K14)</f>
+        <v>3173.59250000001</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <f aca="false">IF(B14+C14=0,"",L14/(B14+C14))</f>
+        <v>634.718500000001</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="9" t="n">
-        <f aca="false">A13*$B$3</f>
-        <v>44900</v>
-      </c>
-      <c r="C13" s="9" t="n">
-        <f aca="false">A13*($B$4+Параметры!$B$3)</f>
-        <v>34150</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <f aca="false">A13*$B$5*$B$3*Параметры!$B$6</f>
-        <v>1459.25</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <f aca="false">A13*(1-$B$5)*$B$3*Параметры!$B$10</f>
-        <v>157.15</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <f aca="false">A13*Параметры!$B$7</f>
+      <c r="D15" s="9" t="n">
+        <f aca="false">B15*$B$4+C15*$C$4</f>
+        <v>99900</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <f aca="false">B15*($B$5+Параметры!$B$3)+C15*($C$5+Параметры!$B$3)</f>
+        <v>71062.3</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <f aca="false">$B$6*D15*Параметры!$B$6</f>
+        <v>3246.75</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <f aca="false">(1-$B$6)*D15*Параметры!$B$10</f>
+        <v>349.65</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <f aca="false">(B15+C15)*Параметры!$B$7</f>
         <v>1800</v>
       </c>
-      <c r="G13" s="9" t="n">
-        <f aca="false">A13*$B$4*Параметры!$B$8</f>
-        <v>1682.5</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <f aca="false">A13*(1-$B$5)*Параметры!$B$11</f>
-        <v>0</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <f aca="false">$B$8</f>
+      <c r="I15" s="9" t="n">
+        <f aca="false">(B15*$B$5+C15*$C$5)*Параметры!$B$8</f>
+        <v>3528.115</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <f aca="false">(B15+C15)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <f aca="false">$B$9</f>
         <v>6783</v>
       </c>
-      <c r="J13" s="11" t="n">
-        <f aca="false">B13-SUM(C13:I13)</f>
-        <v>-1131.9</v>
-      </c>
-      <c r="K13" s="9" t="n">
-        <f aca="false">IF(A13=0,"",J13/A13)</f>
-        <v>-113.19</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="n">
+      <c r="L15" s="11" t="n">
+        <f aca="false">D15-SUM(E15:K15)</f>
+        <v>13130.185</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <f aca="false">IF(B15+C15=0,"",L15/(B15+C15))</f>
+        <v>1313.0185</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <f aca="false">B16*$B$4+C16*$C$4</f>
+        <v>149850</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <f aca="false">B16*($B$5+Параметры!$B$3)+C16*($C$5+Параметры!$B$3)</f>
+        <v>106593.45</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <f aca="false">$B$6*D16*Параметры!$B$6</f>
+        <v>4870.125</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <f aca="false">(1-$B$6)*D16*Параметры!$B$10</f>
+        <v>524.475</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <f aca="false">(B16+C16)*Параметры!$B$7</f>
+        <v>2700</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <f aca="false">(B16*$B$5+C16*$C$5)*Параметры!$B$8</f>
+        <v>5292.1725</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <f aca="false">(B16+C16)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <f aca="false">$B$9</f>
+        <v>6783</v>
+      </c>
+      <c r="L16" s="11" t="n">
+        <f aca="false">D16-SUM(E16:K16)</f>
+        <v>23086.7775</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <f aca="false">IF(B16+C16=0,"",L16/(B16+C16))</f>
+        <v>1539.1185</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="B14" s="9" t="n">
-        <f aca="false">A14*$B$3</f>
+      <c r="D17" s="9" t="n">
+        <f aca="false">B17*$B$4+C17*$C$4</f>
+        <v>199800</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <f aca="false">B17*($B$5+Параметры!$B$3)+C17*($C$5+Параметры!$B$3)</f>
+        <v>142124.6</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <f aca="false">$B$6*D17*Параметры!$B$6</f>
+        <v>6493.5</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <f aca="false">(1-$B$6)*D17*Параметры!$B$10</f>
+        <v>699.3</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <f aca="false">(B17+C17)*Параметры!$B$7</f>
+        <v>3600</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <f aca="false">(B17*$B$5+C17*$C$5)*Параметры!$B$8</f>
+        <v>7056.23</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <f aca="false">(B17+C17)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <f aca="false">$B$9</f>
+        <v>6783</v>
+      </c>
+      <c r="L17" s="11" t="n">
+        <f aca="false">D17-SUM(E17:K17)</f>
+        <v>33043.37</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <f aca="false">IF(B17+C17=0,"",L17/(B17+C17))</f>
+        <v>1652.1685</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <f aca="false">B18*$B$4+C18*$C$4</f>
+        <v>299700</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <f aca="false">B18*($B$5+Параметры!$B$3)+C18*($C$5+Параметры!$B$3)</f>
+        <v>213186.9</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <f aca="false">$B$6*D18*Параметры!$B$6</f>
+        <v>9740.25</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <f aca="false">(1-$B$6)*D18*Параметры!$B$10</f>
+        <v>1048.95</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <f aca="false">(B18+C18)*Параметры!$B$7</f>
+        <v>5400</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <f aca="false">(B18*$B$5+C18*$C$5)*Параметры!$B$8</f>
+        <v>10584.345</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <f aca="false">(B18+C18)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <f aca="false">$B$9</f>
+        <v>6783</v>
+      </c>
+      <c r="L18" s="11" t="n">
+        <f aca="false">D18-SUM(E18:K18)</f>
+        <v>52956.555</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <f aca="false">IF(B18+C18=0,"",L18/(B18+C18))</f>
+        <v>1765.2185</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <f aca="false">B19*$B$4+C19*$C$4</f>
         <v>89800</v>
       </c>
-      <c r="C14" s="9" t="n">
-        <f aca="false">A14*($B$4+Параметры!$B$3)</f>
+      <c r="E19" s="9" t="n">
+        <f aca="false">B19*($B$5+Параметры!$B$3)+C19*($C$5+Параметры!$B$3)</f>
         <v>68300</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <f aca="false">A14*$B$5*$B$3*Параметры!$B$6</f>
+      <c r="F19" s="9" t="n">
+        <f aca="false">$B$6*D19*Параметры!$B$6</f>
         <v>2918.5</v>
       </c>
-      <c r="E14" s="9" t="n">
-        <f aca="false">A14*(1-$B$5)*$B$3*Параметры!$B$10</f>
+      <c r="G19" s="9" t="n">
+        <f aca="false">(1-$B$6)*D19*Параметры!$B$10</f>
         <v>314.3</v>
       </c>
-      <c r="F14" s="9" t="n">
-        <f aca="false">A14*Параметры!$B$7</f>
+      <c r="H19" s="9" t="n">
+        <f aca="false">(B19+C19)*Параметры!$B$7</f>
         <v>3600</v>
       </c>
-      <c r="G14" s="9" t="n">
-        <f aca="false">A14*$B$4*Параметры!$B$8</f>
+      <c r="I19" s="9" t="n">
+        <f aca="false">(B19*$B$5+C19*$C$5)*Параметры!$B$8</f>
         <v>3365</v>
       </c>
-      <c r="H14" s="9" t="n">
-        <f aca="false">A14*(1-$B$5)*Параметры!$B$11</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="9" t="n">
-        <f aca="false">$B$8</f>
+      <c r="J19" s="9" t="n">
+        <f aca="false">(B19+C19)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="9" t="n">
+        <f aca="false">$B$9</f>
         <v>6783</v>
       </c>
-      <c r="J14" s="11" t="n">
-        <f aca="false">B14-SUM(C14:I14)</f>
+      <c r="L19" s="11" t="n">
+        <f aca="false">D19-SUM(E19:K19)</f>
         <v>4519.2</v>
       </c>
-      <c r="K14" s="9" t="n">
-        <f aca="false">IF(A14=0,"",J14/A14)</f>
+      <c r="M19" s="9" t="n">
+        <f aca="false">IF(B19+C19=0,"",L19/(B19+C19))</f>
         <v>225.96</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <f aca="false">B20*$B$4+C20*$C$4</f>
+        <v>139750</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <f aca="false">B20*($B$5+Параметры!$B$3)+C20*($C$5+Параметры!$B$3)</f>
+        <v>103831.15</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <f aca="false">$B$6*D20*Параметры!$B$6</f>
+        <v>4541.875</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <f aca="false">(1-$B$6)*D20*Параметры!$B$10</f>
+        <v>489.125</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <f aca="false">(B20+C20)*Параметры!$B$7</f>
+        <v>4500</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <f aca="false">(B20*$B$5+C20*$C$5)*Параметры!$B$8</f>
+        <v>5129.0575</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <f aca="false">(B20+C20)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <f aca="false">$B$9</f>
+        <v>6783</v>
+      </c>
+      <c r="L20" s="11" t="n">
+        <f aca="false">D20-SUM(E20:K20)</f>
+        <v>14475.7925</v>
+      </c>
+      <c r="M20" s="9" t="n">
+        <f aca="false">IF(B20+C20=0,"",L20/(B20+C20))</f>
+        <v>579.031700000001</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B21" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <f aca="false">B21*$B$4+C21*$C$4</f>
+        <v>189700</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <f aca="false">B21*($B$5+Параметры!$B$3)+C21*($C$5+Параметры!$B$3)</f>
+        <v>139362.3</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <f aca="false">$B$6*D21*Параметры!$B$6</f>
+        <v>6165.25</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <f aca="false">(1-$B$6)*D21*Параметры!$B$10</f>
+        <v>663.95</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <f aca="false">(B21+C21)*Параметры!$B$7</f>
+        <v>5400</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <f aca="false">(B21*$B$5+C21*$C$5)*Параметры!$B$8</f>
+        <v>6893.115</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <f aca="false">(B21+C21)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="9" t="n">
+        <f aca="false">$B$9</f>
+        <v>6783</v>
+      </c>
+      <c r="L21" s="11" t="n">
+        <f aca="false">D21-SUM(E21:K21)</f>
+        <v>24432.385</v>
+      </c>
+      <c r="M21" s="9" t="n">
+        <f aca="false">IF(B21+C21=0,"",L21/(B21+C21))</f>
+        <v>814.412833333334</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B22" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="B15" s="9" t="n">
-        <f aca="false">A15*$B$3</f>
-        <v>134700</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <f aca="false">A15*($B$4+Параметры!$B$3)</f>
-        <v>102450</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <f aca="false">A15*$B$5*$B$3*Параметры!$B$6</f>
-        <v>4377.75</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <f aca="false">A15*(1-$B$5)*$B$3*Параметры!$B$10</f>
-        <v>471.45</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <f aca="false">A15*Параметры!$B$7</f>
-        <v>5400</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <f aca="false">A15*$B$4*Параметры!$B$8</f>
-        <v>5047.5</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <f aca="false">A15*(1-$B$5)*Параметры!$B$11</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <f aca="false">$B$8</f>
+      <c r="C22" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <f aca="false">B22*$B$4+C22*$C$4</f>
+        <v>284550</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <f aca="false">B22*($B$5+Параметры!$B$3)+C22*($C$5+Параметры!$B$3)</f>
+        <v>209043.45</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <f aca="false">$B$6*D22*Параметры!$B$6</f>
+        <v>9247.875</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <f aca="false">(1-$B$6)*D22*Параметры!$B$10</f>
+        <v>995.925</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <f aca="false">(B22+C22)*Параметры!$B$7</f>
+        <v>8100</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <f aca="false">(B22*$B$5+C22*$C$5)*Параметры!$B$8</f>
+        <v>10339.6725</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <f aca="false">(B22+C22)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <f aca="false">$B$9</f>
         <v>6783</v>
       </c>
-      <c r="J15" s="11" t="n">
-        <f aca="false">B15-SUM(C15:I15)</f>
-        <v>10170.3</v>
-      </c>
-      <c r="K15" s="9" t="n">
-        <f aca="false">IF(A15=0,"",J15/A15)</f>
-        <v>339.01</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="n">
+      <c r="L22" s="11" t="n">
+        <f aca="false">D22-SUM(E22:K22)</f>
+        <v>40040.0775</v>
+      </c>
+      <c r="M22" s="9" t="n">
+        <f aca="false">IF(B22+C22=0,"",L22/(B22+C22))</f>
+        <v>889.7795</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B23" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="B16" s="9" t="n">
-        <f aca="false">A16*$B$3</f>
-        <v>224500</v>
-      </c>
-      <c r="C16" s="9" t="n">
-        <f aca="false">A16*($B$4+Параметры!$B$3)</f>
-        <v>170750</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <f aca="false">A16*$B$5*$B$3*Параметры!$B$6</f>
-        <v>7296.25</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <f aca="false">A16*(1-$B$5)*$B$3*Параметры!$B$10</f>
-        <v>785.75</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <f aca="false">A16*Параметры!$B$7</f>
-        <v>9000</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <f aca="false">A16*$B$4*Параметры!$B$8</f>
-        <v>8412.5</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <f aca="false">A16*(1-$B$5)*Параметры!$B$11</f>
-        <v>0</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <f aca="false">$B$8</f>
+      <c r="C23" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <f aca="false">B23*$B$4+C23*$C$4</f>
+        <v>424300</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <f aca="false">B23*($B$5+Параметры!$B$3)+C23*($C$5+Параметры!$B$3)</f>
+        <v>312874.6</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <f aca="false">$B$6*D23*Параметры!$B$6</f>
+        <v>13789.75</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <f aca="false">(1-$B$6)*D23*Параметры!$B$10</f>
+        <v>1485.05</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <f aca="false">(B23+C23)*Параметры!$B$7</f>
+        <v>12600</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <f aca="false">(B23*$B$5+C23*$C$5)*Параметры!$B$8</f>
+        <v>15468.73</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <f aca="false">(B23+C23)*(1-$B$6)*Параметры!$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <f aca="false">$B$9</f>
         <v>6783</v>
       </c>
-      <c r="J16" s="11" t="n">
-        <f aca="false">B16-SUM(C16:I16)</f>
-        <v>21472.5</v>
-      </c>
-      <c r="K16" s="9" t="n">
-        <f aca="false">IF(A16=0,"",J16/A16)</f>
-        <v>429.45</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="B17" s="9" t="n">
-        <f aca="false">A17*$B$3</f>
-        <v>449000</v>
-      </c>
-      <c r="C17" s="9" t="n">
-        <f aca="false">A17*($B$4+Параметры!$B$3)</f>
-        <v>341500</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <f aca="false">A17*$B$5*$B$3*Параметры!$B$6</f>
-        <v>14592.5</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <f aca="false">A17*(1-$B$5)*$B$3*Параметры!$B$10</f>
-        <v>1571.5</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <f aca="false">A17*Параметры!$B$7</f>
-        <v>18000</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <f aca="false">A17*$B$4*Параметры!$B$8</f>
-        <v>16825</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <f aca="false">A17*(1-$B$5)*Параметры!$B$11</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <f aca="false">$B$8</f>
-        <v>6783</v>
-      </c>
-      <c r="J17" s="11" t="n">
-        <f aca="false">B17-SUM(C17:I17)</f>
-        <v>49728</v>
-      </c>
-      <c r="K17" s="9" t="n">
-        <f aca="false">IF(A17=0,"",J17/A17)</f>
-        <v>497.28</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>170</v>
+      <c r="L23" s="11" t="n">
+        <f aca="false">D23-SUM(E23:K23)</f>
+        <v>61298.87</v>
+      </c>
+      <c r="M23" s="9" t="n">
+        <f aca="false">IF(B23+C23=0,"",L23/(B23+C23))</f>
+        <v>875.698142857143</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="C3:J3"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="C8:J8"/>
+  <mergeCells count="6">
+    <mergeCell ref="D3:L3"/>
+    <mergeCell ref="D4:L4"/>
+    <mergeCell ref="D5:L5"/>
+    <mergeCell ref="D6:L6"/>
+    <mergeCell ref="D9:L9"/>
+    <mergeCell ref="D11:L11"/>
   </mergeCells>
-  <conditionalFormatting sqref="J13:J17">
+  <conditionalFormatting sqref="L14:L23">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -4489,206 +4866,206 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B2" s="18" t="n">
         <v>0.3</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>50</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>100</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0.065</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>180</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>0.05</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="B9" s="19" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>0.007</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>4783</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>1500</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>500</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="B17" s="19" t="n">
         <v>20</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">($B$12+$B$13+$B$14+$B$15+$B$16)/MAX(1,$B$17)</f>
         <v>339.15</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -4731,75 +5108,75 @@
         <v>16</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D2" s="22" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="G2" s="23" t="n">
         <v>460</v>
@@ -4831,7 +5208,7 @@
         <v>430</v>
       </c>
       <c r="S2" s="25" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4843,7 +5220,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>1</v>
@@ -4872,7 +5249,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4884,7 +5261,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D4" s="14" t="n">
         <v>1</v>
@@ -4923,7 +5300,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>1</v>
@@ -4962,7 +5339,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>1</v>
@@ -5001,7 +5378,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>1</v>
@@ -5040,7 +5417,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D8" s="14" t="n">
         <v>1</v>
@@ -5069,7 +5446,7 @@
         <v>0</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5081,7 +5458,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>1</v>
@@ -5120,7 +5497,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>1</v>
@@ -5159,7 +5536,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>1</v>
@@ -5198,7 +5575,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>1</v>
@@ -5237,7 +5614,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>1</v>
@@ -5266,7 +5643,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5278,7 +5655,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D14" s="14" t="n">
         <v>1</v>
@@ -5317,7 +5694,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>1</v>
@@ -5356,7 +5733,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>1</v>
@@ -5395,7 +5772,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>1</v>
@@ -5434,7 +5811,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>1</v>
@@ -5463,7 +5840,7 @@
         <v>0</v>
       </c>
       <c r="S18" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5475,7 +5852,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>1</v>
@@ -5514,7 +5891,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D20" s="14" t="n">
         <v>1</v>
@@ -5553,7 +5930,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D21" s="14" t="n">
         <v>1</v>
@@ -5592,7 +5969,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D22" s="14" t="n">
         <v>1</v>
@@ -5631,7 +6008,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D23" s="14" t="n">
         <v>1</v>
@@ -5660,7 +6037,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5672,7 +6049,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D24" s="14" t="n">
         <v>1</v>
@@ -5711,7 +6088,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D25" s="14" t="n">
         <v>1</v>
@@ -5750,7 +6127,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D26" s="14" t="n">
         <v>1</v>
@@ -5789,7 +6166,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D27" s="14" t="n">
         <v>1</v>
@@ -5828,7 +6205,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D28" s="14" t="n">
         <v>1</v>
@@ -5857,7 +6234,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5869,7 +6246,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D29" s="14" t="n">
         <v>1</v>
@@ -5908,7 +6285,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D30" s="14" t="n">
         <v>1</v>
@@ -5947,7 +6324,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D31" s="14" t="n">
         <v>1</v>
@@ -5986,7 +6363,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D32" s="14" t="n">
         <v>1</v>
@@ -6025,7 +6402,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D33" s="14" t="n">
         <v>1</v>
@@ -6054,7 +6431,7 @@
         <v>0</v>
       </c>
       <c r="S33" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6066,7 +6443,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D34" s="14" t="n">
         <v>0</v>
@@ -6095,7 +6472,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="8" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6107,7 +6484,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D35" s="14" t="n">
         <v>1</v>
@@ -6146,7 +6523,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>1</v>
@@ -6185,7 +6562,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D37" s="14" t="n">
         <v>1</v>
@@ -6224,7 +6601,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D38" s="14" t="n">
         <v>1</v>
@@ -6263,7 +6640,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D39" s="14" t="n">
         <v>1</v>
@@ -6292,7 +6669,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6304,7 +6681,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>0</v>
@@ -6333,7 +6710,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="8" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6345,7 +6722,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D41" s="14" t="n">
         <v>1</v>
@@ -6384,7 +6761,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D42" s="14" t="n">
         <v>1</v>
@@ -6423,7 +6800,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D43" s="14" t="n">
         <v>1</v>
@@ -6462,7 +6839,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D44" s="14" t="n">
         <v>1</v>
@@ -6501,7 +6878,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D45" s="14" t="n">
         <v>1</v>
@@ -6530,7 +6907,7 @@
         <v>0</v>
       </c>
       <c r="S45" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6542,7 +6919,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D46" s="14" t="n">
         <v>0</v>
@@ -6571,7 +6948,7 @@
         <v>0</v>
       </c>
       <c r="S46" s="8" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6583,7 +6960,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D47" s="14" t="n">
         <v>1</v>
@@ -6622,7 +6999,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D48" s="14" t="n">
         <v>1</v>
@@ -6661,7 +7038,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D49" s="14" t="n">
         <v>1</v>
@@ -6700,7 +7077,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D50" s="14" t="n">
         <v>1</v>
@@ -6739,7 +7116,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D51" s="14" t="n">
         <v>1</v>
@@ -6768,7 +7145,7 @@
         <v>0</v>
       </c>
       <c r="S51" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6780,7 +7157,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D52" s="14" t="n">
         <v>0</v>
@@ -6809,7 +7186,7 @@
         <v>0</v>
       </c>
       <c r="S52" s="8" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6821,7 +7198,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D53" s="14" t="n">
         <v>1</v>
@@ -6860,7 +7237,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D54" s="14" t="n">
         <v>1</v>
@@ -6899,7 +7276,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D55" s="14" t="n">
         <v>1</v>
@@ -6938,7 +7315,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D56" s="14" t="n">
         <v>1</v>
@@ -6977,7 +7354,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D57" s="14" t="n">
         <v>1</v>
@@ -7006,7 +7383,7 @@
         <v>0</v>
       </c>
       <c r="S57" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7018,7 +7395,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D58" s="14" t="n">
         <v>0</v>
@@ -7047,7 +7424,7 @@
         <v>0</v>
       </c>
       <c r="S58" s="8" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7059,7 +7436,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D59" s="14" t="n">
         <v>1</v>
@@ -7098,7 +7475,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D60" s="14" t="n">
         <v>1</v>
@@ -7137,7 +7514,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D61" s="14" t="n">
         <v>1</v>
@@ -7176,7 +7553,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D62" s="14" t="n">
         <v>1</v>
@@ -7215,7 +7592,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D63" s="14" t="n">
         <v>1</v>
@@ -7244,7 +7621,7 @@
         <v>0</v>
       </c>
       <c r="S63" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7256,7 +7633,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D64" s="14" t="n">
         <v>0</v>
@@ -7285,7 +7662,7 @@
         <v>0</v>
       </c>
       <c r="S64" s="8" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7297,7 +7674,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D65" s="14" t="n">
         <v>1</v>
@@ -7336,7 +7713,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D66" s="14" t="n">
         <v>1</v>
@@ -7375,7 +7752,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D67" s="14" t="n">
         <v>1</v>
@@ -7414,7 +7791,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="D68" s="14" t="n">
         <v>1</v>
@@ -7453,13 +7830,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D69" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="F69" s="14"/>
       <c r="G69" s="12"/>
@@ -7484,7 +7861,7 @@
         <v>0</v>
       </c>
       <c r="S69" s="8" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7496,13 +7873,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D70" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="F70" s="14"/>
       <c r="G70" s="12"/>
@@ -7527,7 +7904,7 @@
         <v>0</v>
       </c>
       <c r="S70" s="8" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7539,13 +7916,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D71" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E71" s="14" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="F71" s="14"/>
       <c r="G71" s="12"/>
@@ -7570,7 +7947,7 @@
         <v>0</v>
       </c>
       <c r="S71" s="8" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7582,13 +7959,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D72" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="F72" s="14"/>
       <c r="G72" s="12"/>
@@ -7613,7 +7990,7 @@
         <v>0</v>
       </c>
       <c r="S72" s="8" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7625,13 +8002,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D73" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="14" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="F73" s="14"/>
       <c r="G73" s="12"/>
@@ -7656,7 +8033,7 @@
         <v>0</v>
       </c>
       <c r="S73" s="8" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7668,13 +8045,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="D74" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="F74" s="14"/>
       <c r="G74" s="12"/>
@@ -7699,7 +8076,7 @@
         <v>0</v>
       </c>
       <c r="S74" s="8" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7711,13 +8088,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="D75" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E75" s="14" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="F75" s="14"/>
       <c r="G75" s="12"/>
@@ -7742,7 +8119,7 @@
         <v>0</v>
       </c>
       <c r="S75" s="8" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7754,13 +8131,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D76" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="F76" s="14"/>
       <c r="G76" s="12"/>
@@ -7785,7 +8162,7 @@
         <v>0</v>
       </c>
       <c r="S76" s="8" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7797,7 +8174,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D77" s="14" t="n">
         <v>1</v>
@@ -7826,7 +8203,7 @@
         <v>0</v>
       </c>
       <c r="S77" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7838,7 +8215,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D78" s="14" t="n">
         <v>1</v>
@@ -7877,7 +8254,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D79" s="14" t="n">
         <v>1</v>
@@ -7916,7 +8293,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D80" s="14" t="n">
         <v>0</v>
@@ -7945,7 +8322,7 @@
         <v>0</v>
       </c>
       <c r="S80" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7957,7 +8334,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D81" s="14" t="n">
         <v>0</v>
@@ -7986,7 +8363,7 @@
         <v>0</v>
       </c>
       <c r="S81" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7998,7 +8375,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D82" s="14" t="n">
         <v>1</v>
@@ -8027,7 +8404,7 @@
         <v>0</v>
       </c>
       <c r="S82" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8039,7 +8416,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D83" s="14" t="n">
         <v>1</v>
@@ -8078,7 +8455,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D84" s="14" t="n">
         <v>1</v>
@@ -8117,7 +8494,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D85" s="14" t="n">
         <v>0</v>
@@ -8146,7 +8523,7 @@
         <v>0</v>
       </c>
       <c r="S85" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8158,7 +8535,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D86" s="14" t="n">
         <v>0</v>
@@ -8187,7 +8564,7 @@
         <v>0</v>
       </c>
       <c r="S86" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8199,7 +8576,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D87" s="14" t="n">
         <v>1</v>
@@ -8228,7 +8605,7 @@
         <v>0</v>
       </c>
       <c r="S87" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8240,7 +8617,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D88" s="14" t="n">
         <v>1</v>
@@ -8279,7 +8656,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D89" s="14" t="n">
         <v>1</v>
@@ -8318,7 +8695,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D90" s="14" t="n">
         <v>0</v>
@@ -8347,7 +8724,7 @@
         <v>0</v>
       </c>
       <c r="S90" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8359,7 +8736,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D91" s="14" t="n">
         <v>0</v>
@@ -8388,7 +8765,7 @@
         <v>0</v>
       </c>
       <c r="S91" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8400,7 +8777,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D92" s="14" t="n">
         <v>1</v>
@@ -8429,7 +8806,7 @@
         <v>0</v>
       </c>
       <c r="S92" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8441,7 +8818,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D93" s="14" t="n">
         <v>1</v>
@@ -8480,7 +8857,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D94" s="14" t="n">
         <v>1</v>
@@ -8519,7 +8896,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D95" s="14" t="n">
         <v>0</v>
@@ -8548,7 +8925,7 @@
         <v>0</v>
       </c>
       <c r="S95" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8560,7 +8937,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D96" s="14" t="n">
         <v>0</v>
@@ -8589,7 +8966,7 @@
         <v>0</v>
       </c>
       <c r="S96" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8601,7 +8978,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D97" s="14" t="n">
         <v>1</v>
@@ -8630,7 +9007,7 @@
         <v>0</v>
       </c>
       <c r="S97" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8642,7 +9019,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D98" s="14" t="n">
         <v>1</v>
@@ -8681,7 +9058,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D99" s="14" t="n">
         <v>1</v>
@@ -8720,7 +9097,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D100" s="14" t="n">
         <v>0</v>
@@ -8749,7 +9126,7 @@
         <v>0</v>
       </c>
       <c r="S100" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8761,7 +9138,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D101" s="14" t="n">
         <v>0</v>
@@ -8790,7 +9167,7 @@
         <v>0</v>
       </c>
       <c r="S101" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8802,7 +9179,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="D102" s="14" t="n">
         <v>1</v>
@@ -8841,7 +9218,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D103" s="14" t="n">
         <v>0</v>
@@ -8870,7 +9247,7 @@
         <v>0</v>
       </c>
       <c r="S103" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8882,7 +9259,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D104" s="14" t="n">
         <v>0</v>
@@ -8911,7 +9288,7 @@
         <v>0</v>
       </c>
       <c r="S104" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8923,7 +9300,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D105" s="14" t="n">
         <v>1</v>
@@ -8952,7 +9329,7 @@
         <v>0</v>
       </c>
       <c r="S105" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8964,7 +9341,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D106" s="14" t="n">
         <v>1</v>
@@ -9003,7 +9380,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D107" s="14" t="n">
         <v>1</v>
@@ -9042,7 +9419,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D108" s="14" t="n">
         <v>0</v>
@@ -9071,7 +9448,7 @@
         <v>0</v>
       </c>
       <c r="S108" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9083,7 +9460,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D109" s="14" t="n">
         <v>0</v>
@@ -9112,7 +9489,7 @@
         <v>0</v>
       </c>
       <c r="S109" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9124,7 +9501,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D110" s="14" t="n">
         <v>1</v>
@@ -9153,7 +9530,7 @@
         <v>0</v>
       </c>
       <c r="S110" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9165,7 +9542,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D111" s="14" t="n">
         <v>1</v>
@@ -9204,7 +9581,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D112" s="14" t="n">
         <v>1</v>
@@ -9243,7 +9620,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D113" s="14" t="n">
         <v>0</v>
@@ -9272,7 +9649,7 @@
         <v>0</v>
       </c>
       <c r="S113" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9284,7 +9661,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D114" s="14" t="n">
         <v>0</v>
@@ -9313,7 +9690,7 @@
         <v>0</v>
       </c>
       <c r="S114" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9325,7 +9702,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D115" s="14" t="n">
         <v>1</v>
@@ -9354,7 +9731,7 @@
         <v>0</v>
       </c>
       <c r="S115" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9366,7 +9743,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D116" s="14" t="n">
         <v>1</v>
@@ -9405,7 +9782,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D117" s="14" t="n">
         <v>1</v>
@@ -9444,7 +9821,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D118" s="14" t="n">
         <v>0</v>
@@ -9473,7 +9850,7 @@
         <v>0</v>
       </c>
       <c r="S118" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9485,7 +9862,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D119" s="14" t="n">
         <v>0</v>
@@ -9514,7 +9891,7 @@
         <v>0</v>
       </c>
       <c r="S119" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9526,7 +9903,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="D120" s="14" t="n">
         <v>1</v>
@@ -9555,7 +9932,7 @@
         <v>0</v>
       </c>
       <c r="S120" s="8" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9567,7 +9944,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="D121" s="14" t="n">
         <v>1</v>
@@ -9606,7 +9983,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D122" s="14" t="n">
         <v>1</v>
@@ -9645,7 +10022,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D123" s="14" t="n">
         <v>0</v>
@@ -9674,7 +10051,7 @@
         <v>0</v>
       </c>
       <c r="S123" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9686,7 +10063,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D124" s="14" t="n">
         <v>0</v>
@@ -9715,7 +10092,7 @@
         <v>0</v>
       </c>
       <c r="S124" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9727,16 +10104,16 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C125" s="7" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="D125" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E125" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="F125" s="14" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="G125" s="12"/>
       <c r="H125" s="12"/>
@@ -9760,7 +10137,7 @@
         <v>0</v>
       </c>
       <c r="S125" s="8" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9772,7 +10149,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C126" s="7" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="D126" s="14" t="n">
         <v>1</v>
@@ -9801,7 +10178,7 @@
         <v>0</v>
       </c>
       <c r="S126" s="8" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9813,7 +10190,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C127" s="7" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D127" s="14" t="n">
         <v>0</v>
@@ -9842,7 +10219,7 @@
         <v>0</v>
       </c>
       <c r="S127" s="8" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9854,7 +10231,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C128" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D128" s="14" t="n">
         <v>0</v>
@@ -9883,7 +10260,7 @@
         <v>0</v>
       </c>
       <c r="S128" s="8" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -9920,80 +10297,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>37</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="E2" s="20" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -10007,10 +10384,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
@@ -10024,10 +10401,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
@@ -10041,10 +10418,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -10058,10 +10435,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
@@ -10075,10 +10452,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
@@ -10092,10 +10469,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
@@ -10109,10 +10486,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -10126,10 +10503,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -10180,7 +10557,7 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>17</v>
@@ -10189,197 +10566,197 @@
         <v>18</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>99</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Brake kits: Kia Rio 4 and Hyundai Solaris 2017+, market price 4 790 ₽
- New kit type «ТОРМОЗ-КИТ» (TRM): front discs AMD AMDBD262 ×2 (2 711,80 ₽
  a pair), pads AMD AMDBF453 (815,10 ₽), caliper guide grease (price TBD)
- AMDBF453 pads are 2017+ (Solaris II / Rio IV), so the kit targets those;
  both articles are listed for Solaris II and Rio IV, hence two listings
- Price set by retail: pair of discs ≈3 540 ₽ + pads ≈1 020 ₽ + grease
- Listing texts, photos, repair cards; workbook handles items without a
  price yet and shows the kit type «Тормоза»; docs updated to 27 kits

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -103,12 +103,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="Y27" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Цена по рынку (сентябрь 2026): диск AMDBD262 в рознице 1 435–2 078 ₽ за штуку (обычно ≈1 770), колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020). Пара дисков + колодки + смазка по отдельности ≈ 4 700 ₽.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y28" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Цена по рынку (сентябрь 2026): диск AMDBD262 в рознице 1 435–2 078 ₽ за штуку (обычно ≈1 770), колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020). Пара дисков + колодки + смазка по отдельности ≈ 4 700 ₽.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="349">
   <si>
     <t xml:space="preserve">ZAPKIT — таблица закупки и цен</t>
   </si>
@@ -560,6 +584,30 @@
     <t xml:space="preserve">grm-12-coolray-1-main.png</t>
   </si>
   <si>
+    <t xml:space="preserve">TRM-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тормоза</t>
+  </si>
+  <si>
+    <t xml:space="preserve">все моторы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тормоз-кит Kia Rio 4 2017–2021: диски и колодки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trm-01-rio-4-1-main.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRM-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тормоз-кит Hyundai Solaris 2017+: диски, колодки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trm-02-solaris-2017-1-main.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Прогноз на месяц (до налога): ТО-киты и ГРМ-киты</t>
   </si>
   <si>
@@ -936,6 +984,30 @@
   </si>
   <si>
     <t xml:space="preserve">Ваша закупка: 990,23 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Диски тормозные передние AMD (AMDBD262) — 2 шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMDBD262</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 2 711,80 ₽ — впишите в колонку поставщика, у которого брали. Цена за пару: кол-во 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Колодки тормозные передние AMD (AMDBF453)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMDBF453</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ваша закупка: 815,10 ₽ — впишите в колонку поставщика, у которого брали</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Смазка для направляющих суппорта</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цены пока нет — впишите в колонку поставщика, у которого берёте</t>
   </si>
   <si>
     <t xml:space="preserve">Поставщик</t>
@@ -1764,7 +1836,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -4045,29 +4117,207 @@
         <v>9990</v>
       </c>
     </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I27" s="9" t="str">
+        <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A27)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="10" t="n">
+        <f aca="false">COUNTIFS(Состав!$A:$A,A27,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
+        <v>3</v>
+      </c>
+      <c r="K27" s="9" t="str">
+        <f aca="false">IF(I27="","",Параметры!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L27" s="9" t="str">
+        <f aca="false">IF(I27="","",I27+K27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="11" t="str">
+        <f aca="false">IF(I27="","",IF(Y27&lt;&gt;"",Y27,CEILING((I27*(1+Параметры!$B$8*Параметры!$B$9)+K27)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))</f>
+        <v/>
+      </c>
+      <c r="N27" s="12"/>
+      <c r="O27" s="7" t="str">
+        <f aca="false">IF(OR(M27="",N27=""),"",IF(M27&lt;=N27,"не дороже рынка","дороже рынка"))</f>
+        <v/>
+      </c>
+      <c r="P27" s="9" t="str">
+        <f aca="false">IF(M27="","",M27*Параметры!$B$6)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="9" t="str">
+        <f aca="false">IF(M27="","",M27*Параметры!$B$10)</f>
+        <v/>
+      </c>
+      <c r="R27" s="9" t="str">
+        <f aca="false">IF(M27="","",Параметры!$B$7)</f>
+        <v/>
+      </c>
+      <c r="S27" s="9" t="str">
+        <f aca="false">IF(I27="","",I27*Параметры!$B$8)</f>
+        <v/>
+      </c>
+      <c r="T27" s="9" t="str">
+        <f aca="false">IF(M27="","",Параметры!$B$18)</f>
+        <v/>
+      </c>
+      <c r="U27" s="11" t="str">
+        <f aca="false">IF(M27="","",M27-L27-P27-R27-S27-T27)</f>
+        <v/>
+      </c>
+      <c r="V27" s="11" t="str">
+        <f aca="false">IF(M27="","",M27-L27-Q27-R27-S27-T27-Параметры!$B$11)</f>
+        <v/>
+      </c>
+      <c r="W27" s="13" t="str">
+        <f aca="false">IF(U27="","",U27/M27)</f>
+        <v/>
+      </c>
+      <c r="X27" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y27" s="12" t="n">
+        <v>4790</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="I28" s="9" t="str">
+        <f aca="false">IF(SUMIFS(Состав!$R:$R,Состав!$A:$A,A28)=0,"",SUMIFS(Состав!$R:$R,Состав!$A:$A,A28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="10" t="n">
+        <f aca="false">COUNTIFS(Состав!$A:$A,A28,Состав!$P:$P,"",Состав!$D:$D,"&gt;0")</f>
+        <v>3</v>
+      </c>
+      <c r="K28" s="9" t="str">
+        <f aca="false">IF(I28="","",Параметры!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L28" s="9" t="str">
+        <f aca="false">IF(I28="","",I28+K28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="11" t="str">
+        <f aca="false">IF(I28="","",IF(Y28&lt;&gt;"",Y28,CEILING((I28*(1+Параметры!$B$8*Параметры!$B$9)+K28)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))</f>
+        <v/>
+      </c>
+      <c r="N28" s="12"/>
+      <c r="O28" s="7" t="str">
+        <f aca="false">IF(OR(M28="",N28=""),"",IF(M28&lt;=N28,"не дороже рынка","дороже рынка"))</f>
+        <v/>
+      </c>
+      <c r="P28" s="9" t="str">
+        <f aca="false">IF(M28="","",M28*Параметры!$B$6)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="9" t="str">
+        <f aca="false">IF(M28="","",M28*Параметры!$B$10)</f>
+        <v/>
+      </c>
+      <c r="R28" s="9" t="str">
+        <f aca="false">IF(M28="","",Параметры!$B$7)</f>
+        <v/>
+      </c>
+      <c r="S28" s="9" t="str">
+        <f aca="false">IF(I28="","",I28*Параметры!$B$8)</f>
+        <v/>
+      </c>
+      <c r="T28" s="9" t="str">
+        <f aca="false">IF(M28="","",Параметры!$B$18)</f>
+        <v/>
+      </c>
+      <c r="U28" s="11" t="str">
+        <f aca="false">IF(M28="","",M28-L28-P28-R28-S28-T28)</f>
+        <v/>
+      </c>
+      <c r="V28" s="11" t="str">
+        <f aca="false">IF(M28="","",M28-L28-Q28-R28-S28-T28-Параметры!$B$11)</f>
+        <v/>
+      </c>
+      <c r="W28" s="13" t="str">
+        <f aca="false">IF(U28="","",U28/M28)</f>
+        <v/>
+      </c>
+      <c r="X28" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y28" s="12" t="n">
+        <v>4790</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J2:J26">
+  <conditionalFormatting sqref="J2:J28">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O26">
+  <conditionalFormatting sqref="O2:O28">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"дороже рынка"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U26">
+  <conditionalFormatting sqref="U2:U28">
     <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V26">
+  <conditionalFormatting sqref="V2:V28">
     <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="X2:X26" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="X2:X28" type="list">
       <formula1>"не выложен,выложен,есть продажи,снят"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4102,19 +4352,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
@@ -4127,7 +4377,7 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>4490</v>
@@ -4136,7 +4386,7 @@
         <v>9990</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
@@ -4149,7 +4399,7 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>3365</v>
@@ -4158,7 +4408,7 @@
         <v>7056.23</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
@@ -4171,13 +4421,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
@@ -4190,7 +4440,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B7" s="9" t="str">
         <f aca="false">IFERROR(AVERAGEIFS(Киты!$M:$M,Киты!$B:$B,"ТО",Киты!$M:$M,"&gt;0"),"")</f>
@@ -4203,7 +4453,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B8" s="9" t="str">
         <f aca="false">IFERROR(AVERAGEIFS(Киты!$I:$I,Киты!$B:$B,"ТО",Киты!$I:$I,"&gt;0"),"")</f>
@@ -4216,14 +4466,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">(Параметры!$B$12+Параметры!$B$13+Параметры!$B$14+Параметры!$B$15+Параметры!$B$16)</f>
         <v>6783</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
@@ -4236,7 +4486,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">B4-(B5+Параметры!$B$3)-$B$6*B4*Параметры!$B$6-(1-$B$6)*(B4*Параметры!$B$10+Параметры!$B$11)-Параметры!$B$7-B5*Параметры!$B$8</f>
@@ -4249,7 +4499,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">IF(B10&lt;=0,"не окупается",ROUNDUP($B$9/B10,0))</f>
@@ -4260,7 +4510,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
@@ -4273,19 +4523,19 @@
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>29</v>
@@ -4300,21 +4550,21 @@
         <v>32</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>0</v>
@@ -4365,7 +4615,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>0</v>
@@ -4416,7 +4666,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B16" s="16" t="n">
         <v>0</v>
@@ -4467,7 +4717,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>0</v>
@@ -4518,7 +4768,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B18" s="16" t="n">
         <v>0</v>
@@ -4569,7 +4819,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B19" s="16" t="n">
         <v>20</v>
@@ -4620,7 +4870,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B20" s="16" t="n">
         <v>20</v>
@@ -4671,7 +4921,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B21" s="16" t="n">
         <v>20</v>
@@ -4722,7 +4972,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B22" s="16" t="n">
         <v>30</v>
@@ -4773,7 +5023,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B23" s="16" t="n">
         <v>50</v>
@@ -4824,7 +5074,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -4866,206 +5116,206 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B2" s="18" t="n">
         <v>0.3</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>50</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>100</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0.065</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>180</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>0.05</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B9" s="19" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>0.007</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>4783</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>1500</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>500</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B17" s="19" t="n">
         <v>20</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">($B$12+$B$13+$B$14+$B$15+$B$16)/MAX(1,$B$17)</f>
         <v>339.15</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -5084,7 +5334,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S128"/>
+  <dimension ref="A1:S134"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -5108,75 +5358,75 @@
         <v>16</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D2" s="22" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="G2" s="23" t="n">
         <v>460</v>
@@ -5208,7 +5458,7 @@
         <v>430</v>
       </c>
       <c r="S2" s="25" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5220,7 +5470,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>1</v>
@@ -5249,7 +5499,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5261,7 +5511,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D4" s="14" t="n">
         <v>1</v>
@@ -5300,7 +5550,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>1</v>
@@ -5339,7 +5589,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>1</v>
@@ -5378,7 +5628,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D7" s="14" t="n">
         <v>1</v>
@@ -5417,7 +5667,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D8" s="14" t="n">
         <v>1</v>
@@ -5446,7 +5696,7 @@
         <v>0</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5458,7 +5708,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>1</v>
@@ -5497,7 +5747,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>1</v>
@@ -5536,7 +5786,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>1</v>
@@ -5575,7 +5825,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>1</v>
@@ -5614,7 +5864,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>1</v>
@@ -5643,7 +5893,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5655,7 +5905,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D14" s="14" t="n">
         <v>1</v>
@@ -5694,7 +5944,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>1</v>
@@ -5733,7 +5983,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>1</v>
@@ -5772,7 +6022,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>1</v>
@@ -5811,7 +6061,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>1</v>
@@ -5840,7 +6090,7 @@
         <v>0</v>
       </c>
       <c r="S18" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5852,7 +6102,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>1</v>
@@ -5891,7 +6141,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D20" s="14" t="n">
         <v>1</v>
@@ -5930,7 +6180,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D21" s="14" t="n">
         <v>1</v>
@@ -5969,7 +6219,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D22" s="14" t="n">
         <v>1</v>
@@ -6008,7 +6258,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D23" s="14" t="n">
         <v>1</v>
@@ -6037,7 +6287,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6049,7 +6299,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D24" s="14" t="n">
         <v>1</v>
@@ -6088,7 +6338,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D25" s="14" t="n">
         <v>1</v>
@@ -6127,7 +6377,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D26" s="14" t="n">
         <v>1</v>
@@ -6166,7 +6416,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D27" s="14" t="n">
         <v>1</v>
@@ -6205,7 +6455,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D28" s="14" t="n">
         <v>1</v>
@@ -6234,7 +6484,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6246,7 +6496,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D29" s="14" t="n">
         <v>1</v>
@@ -6285,7 +6535,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D30" s="14" t="n">
         <v>1</v>
@@ -6324,7 +6574,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D31" s="14" t="n">
         <v>1</v>
@@ -6363,7 +6613,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D32" s="14" t="n">
         <v>1</v>
@@ -6402,7 +6652,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D33" s="14" t="n">
         <v>1</v>
@@ -6431,7 +6681,7 @@
         <v>0</v>
       </c>
       <c r="S33" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6443,7 +6693,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D34" s="14" t="n">
         <v>0</v>
@@ -6472,7 +6722,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6484,7 +6734,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D35" s="14" t="n">
         <v>1</v>
@@ -6523,7 +6773,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>1</v>
@@ -6562,7 +6812,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D37" s="14" t="n">
         <v>1</v>
@@ -6601,7 +6851,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D38" s="14" t="n">
         <v>1</v>
@@ -6640,7 +6890,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D39" s="14" t="n">
         <v>1</v>
@@ -6669,7 +6919,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6681,7 +6931,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>0</v>
@@ -6710,7 +6960,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6722,7 +6972,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D41" s="14" t="n">
         <v>1</v>
@@ -6761,7 +7011,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D42" s="14" t="n">
         <v>1</v>
@@ -6800,7 +7050,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D43" s="14" t="n">
         <v>1</v>
@@ -6839,7 +7089,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D44" s="14" t="n">
         <v>1</v>
@@ -6878,7 +7128,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D45" s="14" t="n">
         <v>1</v>
@@ -6907,7 +7157,7 @@
         <v>0</v>
       </c>
       <c r="S45" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6919,7 +7169,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D46" s="14" t="n">
         <v>0</v>
@@ -6948,7 +7198,7 @@
         <v>0</v>
       </c>
       <c r="S46" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6960,7 +7210,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D47" s="14" t="n">
         <v>1</v>
@@ -6999,7 +7249,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D48" s="14" t="n">
         <v>1</v>
@@ -7038,7 +7288,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D49" s="14" t="n">
         <v>1</v>
@@ -7077,7 +7327,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D50" s="14" t="n">
         <v>1</v>
@@ -7116,7 +7366,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D51" s="14" t="n">
         <v>1</v>
@@ -7145,7 +7395,7 @@
         <v>0</v>
       </c>
       <c r="S51" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7157,7 +7407,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D52" s="14" t="n">
         <v>0</v>
@@ -7186,7 +7436,7 @@
         <v>0</v>
       </c>
       <c r="S52" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7198,7 +7448,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D53" s="14" t="n">
         <v>1</v>
@@ -7237,7 +7487,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D54" s="14" t="n">
         <v>1</v>
@@ -7276,7 +7526,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D55" s="14" t="n">
         <v>1</v>
@@ -7315,7 +7565,7 @@
         <v>Chery Tiggo 7 Pro 1.5T</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D56" s="14" t="n">
         <v>1</v>
@@ -7354,7 +7604,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D57" s="14" t="n">
         <v>1</v>
@@ -7383,7 +7633,7 @@
         <v>0</v>
       </c>
       <c r="S57" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7395,7 +7645,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D58" s="14" t="n">
         <v>0</v>
@@ -7424,7 +7674,7 @@
         <v>0</v>
       </c>
       <c r="S58" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7436,7 +7686,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D59" s="14" t="n">
         <v>1</v>
@@ -7475,7 +7725,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D60" s="14" t="n">
         <v>1</v>
@@ -7514,7 +7764,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D61" s="14" t="n">
         <v>1</v>
@@ -7553,7 +7803,7 @@
         <v>Chery Tiggo 4 Pro 1.5T</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D62" s="14" t="n">
         <v>1</v>
@@ -7592,7 +7842,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D63" s="14" t="n">
         <v>1</v>
@@ -7621,7 +7871,7 @@
         <v>0</v>
       </c>
       <c r="S63" s="8" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7633,7 +7883,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D64" s="14" t="n">
         <v>0</v>
@@ -7662,7 +7912,7 @@
         <v>0</v>
       </c>
       <c r="S64" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7674,7 +7924,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D65" s="14" t="n">
         <v>1</v>
@@ -7713,7 +7963,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D66" s="14" t="n">
         <v>1</v>
@@ -7752,7 +8002,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D67" s="14" t="n">
         <v>1</v>
@@ -7791,7 +8041,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D68" s="14" t="n">
         <v>1</v>
@@ -7830,13 +8080,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D69" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="F69" s="14"/>
       <c r="G69" s="12"/>
@@ -7861,7 +8111,7 @@
         <v>0</v>
       </c>
       <c r="S69" s="8" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7873,13 +8123,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D70" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F70" s="14"/>
       <c r="G70" s="12"/>
@@ -7904,7 +8154,7 @@
         <v>0</v>
       </c>
       <c r="S70" s="8" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7916,13 +8166,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D71" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E71" s="14" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F71" s="14"/>
       <c r="G71" s="12"/>
@@ -7947,7 +8197,7 @@
         <v>0</v>
       </c>
       <c r="S71" s="8" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7959,13 +8209,13 @@
         <v>Kia Picanto 1.0 / 1.2</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D72" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="F72" s="14"/>
       <c r="G72" s="12"/>
@@ -7990,7 +8240,7 @@
         <v>0</v>
       </c>
       <c r="S72" s="8" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8002,13 +8252,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D73" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="14" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="F73" s="14"/>
       <c r="G73" s="12"/>
@@ -8033,7 +8283,7 @@
         <v>0</v>
       </c>
       <c r="S73" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8045,13 +8295,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D74" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F74" s="14"/>
       <c r="G74" s="12"/>
@@ -8076,7 +8326,7 @@
         <v>0</v>
       </c>
       <c r="S74" s="8" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8088,13 +8338,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D75" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E75" s="14" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="F75" s="14"/>
       <c r="G75" s="12"/>
@@ -8119,7 +8369,7 @@
         <v>0</v>
       </c>
       <c r="S75" s="8" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8131,13 +8381,13 @@
         <v>VW Jetta</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D76" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="F76" s="14"/>
       <c r="G76" s="12"/>
@@ -8162,7 +8412,7 @@
         <v>0</v>
       </c>
       <c r="S76" s="8" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8174,7 +8424,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D77" s="14" t="n">
         <v>1</v>
@@ -8203,7 +8453,7 @@
         <v>0</v>
       </c>
       <c r="S77" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8215,7 +8465,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D78" s="14" t="n">
         <v>1</v>
@@ -8254,7 +8504,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D79" s="14" t="n">
         <v>1</v>
@@ -8293,7 +8543,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D80" s="14" t="n">
         <v>0</v>
@@ -8322,7 +8572,7 @@
         <v>0</v>
       </c>
       <c r="S80" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8334,7 +8584,7 @@
         <v>Hyundai Solaris 2010–2017</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D81" s="14" t="n">
         <v>0</v>
@@ -8363,7 +8613,7 @@
         <v>0</v>
       </c>
       <c r="S81" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8375,7 +8625,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D82" s="14" t="n">
         <v>1</v>
@@ -8404,7 +8654,7 @@
         <v>0</v>
       </c>
       <c r="S82" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8416,7 +8666,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D83" s="14" t="n">
         <v>1</v>
@@ -8455,7 +8705,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D84" s="14" t="n">
         <v>1</v>
@@ -8494,7 +8744,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D85" s="14" t="n">
         <v>0</v>
@@ -8523,7 +8773,7 @@
         <v>0</v>
       </c>
       <c r="S85" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8535,7 +8785,7 @@
         <v>Hyundai Solaris 2017–2022</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D86" s="14" t="n">
         <v>0</v>
@@ -8564,7 +8814,7 @@
         <v>0</v>
       </c>
       <c r="S86" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8576,7 +8826,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D87" s="14" t="n">
         <v>1</v>
@@ -8605,7 +8855,7 @@
         <v>0</v>
       </c>
       <c r="S87" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8617,7 +8867,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D88" s="14" t="n">
         <v>1</v>
@@ -8656,7 +8906,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D89" s="14" t="n">
         <v>1</v>
@@ -8695,7 +8945,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D90" s="14" t="n">
         <v>0</v>
@@ -8724,7 +8974,7 @@
         <v>0</v>
       </c>
       <c r="S90" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8736,7 +8986,7 @@
         <v>Kia Rio 2011–2017</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D91" s="14" t="n">
         <v>0</v>
@@ -8765,7 +9015,7 @@
         <v>0</v>
       </c>
       <c r="S91" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8777,7 +9027,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D92" s="14" t="n">
         <v>1</v>
@@ -8806,7 +9056,7 @@
         <v>0</v>
       </c>
       <c r="S92" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8818,7 +9068,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D93" s="14" t="n">
         <v>1</v>
@@ -8857,7 +9107,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D94" s="14" t="n">
         <v>1</v>
@@ -8896,7 +9146,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D95" s="14" t="n">
         <v>0</v>
@@ -8925,7 +9175,7 @@
         <v>0</v>
       </c>
       <c r="S95" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8937,7 +9187,7 @@
         <v>Kia Rio 2017–2021</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D96" s="14" t="n">
         <v>0</v>
@@ -8966,7 +9216,7 @@
         <v>0</v>
       </c>
       <c r="S96" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8978,7 +9228,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D97" s="14" t="n">
         <v>1</v>
@@ -9007,7 +9257,7 @@
         <v>0</v>
       </c>
       <c r="S97" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9019,7 +9269,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D98" s="14" t="n">
         <v>1</v>
@@ -9058,7 +9308,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D99" s="14" t="n">
         <v>1</v>
@@ -9097,7 +9347,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D100" s="14" t="n">
         <v>0</v>
@@ -9126,7 +9376,7 @@
         <v>0</v>
       </c>
       <c r="S100" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9138,7 +9388,7 @@
         <v>VW Polo 1.6 CFNA</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D101" s="14" t="n">
         <v>0</v>
@@ -9167,7 +9417,7 @@
         <v>0</v>
       </c>
       <c r="S101" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9179,7 +9429,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="D102" s="14" t="n">
         <v>1</v>
@@ -9218,7 +9468,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D103" s="14" t="n">
         <v>0</v>
@@ -9247,7 +9497,7 @@
         <v>0</v>
       </c>
       <c r="S103" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9259,7 +9509,7 @@
         <v>VW Polo 1.6 CWVA</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D104" s="14" t="n">
         <v>0</v>
@@ -9288,7 +9538,7 @@
         <v>0</v>
       </c>
       <c r="S104" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9300,7 +9550,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D105" s="14" t="n">
         <v>1</v>
@@ -9329,7 +9579,7 @@
         <v>0</v>
       </c>
       <c r="S105" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9341,7 +9591,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D106" s="14" t="n">
         <v>1</v>
@@ -9380,7 +9630,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D107" s="14" t="n">
         <v>1</v>
@@ -9419,7 +9669,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D108" s="14" t="n">
         <v>0</v>
@@ -9448,7 +9698,7 @@
         <v>0</v>
       </c>
       <c r="S108" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9460,7 +9710,7 @@
         <v>Haval Jolion 1.5T</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D109" s="14" t="n">
         <v>0</v>
@@ -9489,7 +9739,7 @@
         <v>0</v>
       </c>
       <c r="S109" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9501,7 +9751,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D110" s="14" t="n">
         <v>1</v>
@@ -9530,7 +9780,7 @@
         <v>0</v>
       </c>
       <c r="S110" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9542,7 +9792,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D111" s="14" t="n">
         <v>1</v>
@@ -9581,7 +9831,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D112" s="14" t="n">
         <v>1</v>
@@ -9620,7 +9870,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D113" s="14" t="n">
         <v>0</v>
@@ -9649,7 +9899,7 @@
         <v>0</v>
       </c>
       <c r="S113" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9661,7 +9911,7 @@
         <v>Haval F7 / F7x 1.5T</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D114" s="14" t="n">
         <v>0</v>
@@ -9690,7 +9940,7 @@
         <v>0</v>
       </c>
       <c r="S114" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9702,7 +9952,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D115" s="14" t="n">
         <v>1</v>
@@ -9731,7 +9981,7 @@
         <v>0</v>
       </c>
       <c r="S115" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9743,7 +9993,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D116" s="14" t="n">
         <v>1</v>
@@ -9782,7 +10032,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D117" s="14" t="n">
         <v>1</v>
@@ -9821,7 +10071,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D118" s="14" t="n">
         <v>0</v>
@@ -9850,7 +10100,7 @@
         <v>0</v>
       </c>
       <c r="S118" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9862,7 +10112,7 @@
         <v>Haval F7 / F7x 2.0T</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D119" s="14" t="n">
         <v>0</v>
@@ -9891,7 +10141,7 @@
         <v>0</v>
       </c>
       <c r="S119" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9903,7 +10153,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D120" s="14" t="n">
         <v>1</v>
@@ -9932,7 +10182,7 @@
         <v>0</v>
       </c>
       <c r="S120" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9944,7 +10194,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D121" s="14" t="n">
         <v>1</v>
@@ -9983,7 +10233,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D122" s="14" t="n">
         <v>1</v>
@@ -10022,7 +10272,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D123" s="14" t="n">
         <v>0</v>
@@ -10051,7 +10301,7 @@
         <v>0</v>
       </c>
       <c r="S123" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10063,7 +10313,7 @@
         <v>Chery Tiggo 7 Pro / 4 Pro 1.5T</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D124" s="14" t="n">
         <v>0</v>
@@ -10092,7 +10342,7 @@
         <v>0</v>
       </c>
       <c r="S124" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10104,16 +10354,16 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C125" s="7" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="D125" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E125" s="14" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="F125" s="14" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="G125" s="12"/>
       <c r="H125" s="12"/>
@@ -10137,7 +10387,7 @@
         <v>0</v>
       </c>
       <c r="S125" s="8" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10149,7 +10399,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C126" s="7" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="D126" s="14" t="n">
         <v>1</v>
@@ -10178,7 +10428,7 @@
         <v>0</v>
       </c>
       <c r="S126" s="8" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10190,7 +10440,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C127" s="7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D127" s="14" t="n">
         <v>0</v>
@@ -10219,7 +10469,7 @@
         <v>0</v>
       </c>
       <c r="S127" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10231,7 +10481,7 @@
         <v>Geely Coolray 1.5T</v>
       </c>
       <c r="C128" s="7" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D128" s="14" t="n">
         <v>0</v>
@@ -10260,7 +10510,269 @@
         <v>0</v>
       </c>
       <c r="S128" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B129" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A129,Киты!$A:$A,0)),"")</f>
+        <v>Kia Rio 2017–2021</v>
+      </c>
+      <c r="C129" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D129" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E129" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F129" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="G129" s="12"/>
+      <c r="H129" s="12"/>
+      <c r="I129" s="12"/>
+      <c r="J129" s="12"/>
+      <c r="K129" s="12"/>
+      <c r="L129" s="12"/>
+      <c r="M129" s="12"/>
+      <c r="N129" s="12"/>
+      <c r="O129" s="12"/>
+      <c r="P129" s="9" t="str">
+        <f aca="false">IF(COUNT(G129:O129)=0,"",MIN(G129:O129))</f>
+        <v/>
+      </c>
+      <c r="Q129" s="7" t="str">
+        <f aca="false">IF(P129="","",INDEX($G$1:$O$1,MATCH(P129,G129:O129,0)))</f>
+        <v/>
+      </c>
+      <c r="R129" s="9" t="n">
+        <f aca="false">IF(P129="",0,P129*D129)</f>
+        <v>0</v>
+      </c>
+      <c r="S129" s="8" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B130" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A130,Киты!$A:$A,0)),"")</f>
+        <v>Kia Rio 2017–2021</v>
+      </c>
+      <c r="C130" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="D130" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E130" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F130" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="G130" s="12"/>
+      <c r="H130" s="12"/>
+      <c r="I130" s="12"/>
+      <c r="J130" s="12"/>
+      <c r="K130" s="12"/>
+      <c r="L130" s="12"/>
+      <c r="M130" s="12"/>
+      <c r="N130" s="12"/>
+      <c r="O130" s="12"/>
+      <c r="P130" s="9" t="str">
+        <f aca="false">IF(COUNT(G130:O130)=0,"",MIN(G130:O130))</f>
+        <v/>
+      </c>
+      <c r="Q130" s="7" t="str">
+        <f aca="false">IF(P130="","",INDEX($G$1:$O$1,MATCH(P130,G130:O130,0)))</f>
+        <v/>
+      </c>
+      <c r="R130" s="9" t="n">
+        <f aca="false">IF(P130="",0,P130*D130)</f>
+        <v>0</v>
+      </c>
+      <c r="S130" s="8" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B131" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A131,Киты!$A:$A,0)),"")</f>
+        <v>Kia Rio 2017–2021</v>
+      </c>
+      <c r="C131" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="D131" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E131" s="14"/>
+      <c r="F131" s="14"/>
+      <c r="G131" s="12"/>
+      <c r="H131" s="12"/>
+      <c r="I131" s="12"/>
+      <c r="J131" s="12"/>
+      <c r="K131" s="12"/>
+      <c r="L131" s="12"/>
+      <c r="M131" s="12"/>
+      <c r="N131" s="12"/>
+      <c r="O131" s="12"/>
+      <c r="P131" s="9" t="str">
+        <f aca="false">IF(COUNT(G131:O131)=0,"",MIN(G131:O131))</f>
+        <v/>
+      </c>
+      <c r="Q131" s="7" t="str">
+        <f aca="false">IF(P131="","",INDEX($G$1:$O$1,MATCH(P131,G131:O131,0)))</f>
+        <v/>
+      </c>
+      <c r="R131" s="9" t="n">
+        <f aca="false">IF(P131="",0,P131*D131)</f>
+        <v>0</v>
+      </c>
+      <c r="S131" s="8" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B132" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A132,Киты!$A:$A,0)),"")</f>
+        <v>Hyundai Solaris 2017–2022</v>
+      </c>
+      <c r="C132" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D132" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E132" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F132" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="G132" s="12"/>
+      <c r="H132" s="12"/>
+      <c r="I132" s="12"/>
+      <c r="J132" s="12"/>
+      <c r="K132" s="12"/>
+      <c r="L132" s="12"/>
+      <c r="M132" s="12"/>
+      <c r="N132" s="12"/>
+      <c r="O132" s="12"/>
+      <c r="P132" s="9" t="str">
+        <f aca="false">IF(COUNT(G132:O132)=0,"",MIN(G132:O132))</f>
+        <v/>
+      </c>
+      <c r="Q132" s="7" t="str">
+        <f aca="false">IF(P132="","",INDEX($G$1:$O$1,MATCH(P132,G132:O132,0)))</f>
+        <v/>
+      </c>
+      <c r="R132" s="9" t="n">
+        <f aca="false">IF(P132="",0,P132*D132)</f>
+        <v>0</v>
+      </c>
+      <c r="S132" s="8" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B133" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A133,Киты!$A:$A,0)),"")</f>
+        <v>Hyundai Solaris 2017–2022</v>
+      </c>
+      <c r="C133" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="D133" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E133" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F133" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="G133" s="12"/>
+      <c r="H133" s="12"/>
+      <c r="I133" s="12"/>
+      <c r="J133" s="12"/>
+      <c r="K133" s="12"/>
+      <c r="L133" s="12"/>
+      <c r="M133" s="12"/>
+      <c r="N133" s="12"/>
+      <c r="O133" s="12"/>
+      <c r="P133" s="9" t="str">
+        <f aca="false">IF(COUNT(G133:O133)=0,"",MIN(G133:O133))</f>
+        <v/>
+      </c>
+      <c r="Q133" s="7" t="str">
+        <f aca="false">IF(P133="","",INDEX($G$1:$O$1,MATCH(P133,G133:O133,0)))</f>
+        <v/>
+      </c>
+      <c r="R133" s="9" t="n">
+        <f aca="false">IF(P133="",0,P133*D133)</f>
+        <v>0</v>
+      </c>
+      <c r="S133" s="8" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B134" s="7" t="str">
+        <f aca="false">IFERROR(INDEX(Киты!$C:$C,MATCH(A134,Киты!$A:$A,0)),"")</f>
+        <v>Hyundai Solaris 2017–2022</v>
+      </c>
+      <c r="C134" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="D134" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" s="14"/>
+      <c r="F134" s="14"/>
+      <c r="G134" s="12"/>
+      <c r="H134" s="12"/>
+      <c r="I134" s="12"/>
+      <c r="J134" s="12"/>
+      <c r="K134" s="12"/>
+      <c r="L134" s="12"/>
+      <c r="M134" s="12"/>
+      <c r="N134" s="12"/>
+      <c r="O134" s="12"/>
+      <c r="P134" s="9" t="str">
+        <f aca="false">IF(COUNT(G134:O134)=0,"",MIN(G134:O134))</f>
+        <v/>
+      </c>
+      <c r="Q134" s="7" t="str">
+        <f aca="false">IF(P134="","",INDEX($G$1:$O$1,MATCH(P134,G134:O134,0)))</f>
+        <v/>
+      </c>
+      <c r="R134" s="9" t="n">
+        <f aca="false">IF(P134="",0,P134*D134)</f>
+        <v>0</v>
+      </c>
+      <c r="S134" s="8" t="s">
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -10297,80 +10809,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>37</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>280</v>
+        <v>296</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>281</v>
+        <v>297</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>283</v>
+        <v>299</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>284</v>
+        <v>300</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>287</v>
+        <v>303</v>
       </c>
       <c r="E2" s="20" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>288</v>
+        <v>304</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>289</v>
+        <v>305</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>290</v>
+        <v>306</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>291</v>
+        <v>307</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -10384,10 +10896,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
@@ -10401,10 +10913,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
@@ -10418,10 +10930,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -10435,10 +10947,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
@@ -10452,10 +10964,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
@@ -10469,10 +10981,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
@@ -10486,10 +10998,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -10503,10 +11015,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -10557,7 +11069,7 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>17</v>
@@ -10566,197 +11078,197 @@
         <v>18</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>295</v>
+        <v>311</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>296</v>
+        <v>312</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>297</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>300</v>
+        <v>316</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>302</v>
+        <v>318</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>304</v>
+        <v>320</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>305</v>
+        <v>321</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>306</v>
+        <v>322</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>307</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>308</v>
+        <v>324</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>310</v>
+        <v>326</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>307</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>314</v>
+        <v>330</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>307</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>318</v>
+        <v>334</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>320</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>324</v>
+        <v>340</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>325</v>
+        <v>341</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>329</v>
+        <v>345</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>99</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>331</v>
+        <v>347</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>332</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Brake kits: grease 97,70 ₽, price 4 990 ₽ by retail disc prices
- Caliper guide grease bought at 97,70 ₽
- Retail AMD front discs are ≈1 700–2 300 ₽ each, so the same set bought
  separately costs ≈5 150 ₽; the kit is priced at 4 990 ₽

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -111,7 +111,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена по рынку (сентябрь 2026): диск AMDBD262 в рознице 1 435–2 078 ₽ за штуку (обычно ≈1 770), колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020). Пара дисков + колодки + смазка по отдельности ≈ 4 700 ₽.</t>
+          <t xml:space="preserve">Цена по рынку (сентябрь 2026): диск AMD в рознице ≈1 700–2 300 ₽ за штуку, колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020), смазка ≈100–150 ₽. По отдельности покупатель отдаст ≈5 150 ₽ (от 4 300 до 6 000) — у нас дешевле и одной коробкой.</t>
         </r>
       </text>
     </comment>
@@ -123,7 +123,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена по рынку (сентябрь 2026): диск AMDBD262 в рознице 1 435–2 078 ₽ за штуку (обычно ≈1 770), колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020). Пара дисков + колодки + смазка по отдельности ≈ 4 700 ₽.</t>
+          <t xml:space="preserve">Цена по рынку (сентябрь 2026): диск AMD в рознице ≈1 700–2 300 ₽ за штуку, колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020), смазка ≈100–150 ₽. По отдельности покупатель отдаст ≈5 150 ₽ (от 4 300 до 6 000) — у нас дешевле и одной коробкой.</t>
         </r>
       </text>
     </comment>
@@ -1007,7 +1007,7 @@
     <t xml:space="preserve">Смазка для направляющих суппорта</t>
   </si>
   <si>
-    <t xml:space="preserve">Цены пока нет — впишите в колонку поставщика, у которого берёте</t>
+    <t xml:space="preserve">Ваша закупка: 97,70 ₽ — впишите в колонку поставщика, у которого брали</t>
   </si>
   <si>
     <t xml:space="preserve">Поставщик</t>
@@ -4203,7 +4203,7 @@
         <v>47</v>
       </c>
       <c r="Y27" s="12" t="n">
-        <v>4790</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4292,7 +4292,7 @@
         <v>47</v>
       </c>
       <c r="Y28" s="12" t="n">
-        <v>4790</v>
+        <v>4990</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Client loop: decisions on hours, calls, VIN re-check, single parts, pickup
- Working hours 9:00–20:00 every day; calls accepted in those hours,
  VIN still goes to the chat
- Bought without chatting: always re-check by VIN, never ship unchecked,
  cancel if the check cannot be done in time
- Single parts on request, always asking what repair it is for
- Self-pickup in Sochi: transfer in advance, place and time agreed
- Lead sheet: «Оплата и получение» (Авито Доставка / перевод + СДЭК /
  перевод + самовывоз); diagram, listings and store text updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -636,7 +636,7 @@
     <t xml:space="preserve">Сумма, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Оплата</t>
+    <t xml:space="preserve">Оплата и получение</t>
   </si>
   <si>
     <t xml:space="preserve">Причина отказа</t>
@@ -10501,7 +10501,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K3:K302" type="list">
-      <formula1>"Авито Доставка,перевод"</formula1>
+      <formula1>"Авито Доставка,перевод + СДЭК,перевод + самовывоз"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L3:L302" type="list">

</xml_diff>

<commit_message>
Prices right at the market level for the five priced kits
- Market price = typical retail of the same parts elsewhere, rounded down
  to …90: Picanto 4 090, Jetta 4 990, Coolray 10 790, brake kits 5 090 ₽;
  the breakdown is kept in price_note (cell comment on «Киты», column Y)
- A market price is now final: the +5% raise applies only to kits priced
  by markup until their market is checked
- Docs: pricing rule for kits, other brands, single parts and cars not
  in the list; store mockup price for Coolray

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmRinhBKDvaShQvm1XSe1Q
</commit_message>
<xml_diff>
--- a/avito/zapkit-zakupka.xlsx
+++ b/avito/zapkit-zakupka.xlsx
@@ -52,7 +52,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">База — по наценке с листа «Параметры» или цена по рынку из колонки Y, если она есть. Сверху — «Повышение цен» с листа «Параметры», затем округление до …90.</t>
+          <t xml:space="preserve">Если в колонке Y есть цена по рынку — берётся она. Иначе — наценка и повышение цен с листа «Параметры», округление до …90.</t>
         </r>
       </text>
     </comment>
@@ -88,7 +88,31 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Для китов, где цену ставим по рынку, а не по наценке: впишите цену, по которой конечный покупатель берёт то же самое на маркетплейсах. Повышение цен добавится сверху. Пусто — цена по наценке.</t>
+          <t xml:space="preserve">Цена впритык к рынку: сложите типичные розничные цены тех же деталей у других продавцов и округлите вниз до …90. Это и есть цена кита. Пусто — цена по наценке.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Впритык к рынку (сентябрь 2026): масло Hyundai/Kia 5W-30 4 л в рознице 2 187–3 109 ₽ (≈2 650), фильтры AMD масляный ≈300, AMD воздушный ≈700, салонный ≈450 (оценка по похожим позициям). Итого по отдельности ≈4 100 ₽ → 4 090 ₽.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Впритык к рынку (сентябрь 2026): масло Teboil Diamond Multi 5W-40 4 л в рознице 3 290–3 950 ₽ (≈3 675), масляный фильтр AMD ≈350 (309–422), воздушный BRAVE ≈500 и салонный BRAVE ≈450 (оценка, от 410 ₽). Итого по отдельности ≈4 975 ₽ → 4 990 ₽.</t>
         </r>
       </text>
     </comment>
@@ -100,7 +124,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Рыночная база (сентябрь 2026): Gates K0120529 отдельно — 7 290–10 526 ₽ в рознице, ремень помпы — 740–1 679 ₽. Итоговая цена — база плюс повышение с листа «Параметры»; даже с ним кит дешевле, чем Gates и ремень помпы по отдельности на Яндекс Маркете.</t>
+          <t xml:space="preserve">Впритык к рынку (сентябрь 2026): Gates K0120529 в рознице 7 290–14 130 ₽ (типично ≈9 610), ремень помпы 740–1 679 ₽ (≈1 200). Итого по отдельности ≈10 810 ₽ → 10 790 ₽.</t>
         </r>
       </text>
     </comment>
@@ -112,7 +136,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Рыночная база (сентябрь 2026): диск AMD в рознице ≈1 700–2 300 ₽ за штуку, колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020), смазка ≈100–150 ₽. По отдельности покупатель отдаст ≈5 150 ₽ (от 4 300 до 6 000). Итоговая цена — база плюс повышение с листа «Параметры».</t>
+          <t xml:space="preserve">Впритык к рынку (сентябрь 2026): диск AMD ≈1 700–2 300 ₽ за штуку (≈2 000 × 2), колодки AMDBF453 806–1 289 ₽ (≈1 020), смазка ≈100–150 ₽. Итого по отдельности ≈5 145 ₽ → 5 090 ₽.</t>
         </r>
       </text>
     </comment>
@@ -124,7 +148,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Рыночная база (сентябрь 2026): диск AMD в рознице ≈1 700–2 300 ₽ за штуку, колодки AMDBF453 — 806–1 289 ₽ (обычно ≈1 020), смазка ≈100–150 ₽. По отдельности покупатель отдаст ≈5 150 ₽ (от 4 300 до 6 000). Итоговая цена — база плюс повышение с листа «Параметры».</t>
+          <t xml:space="preserve">Впритык к рынку (сентябрь 2026): диск AMD ≈1 700–2 300 ₽ за штуку (≈2 000 × 2), колодки AMDBF453 806–1 289 ₽ (≈1 020), смазка ≈100–150 ₽. Итого по отдельности ≈5 145 ₽ → 5 090 ₽.</t>
         </r>
       </text>
     </comment>
@@ -153,7 +177,7 @@
     <t xml:space="preserve">3. «Киты» — сами посчитаются закупка, цена на Авито и прибыль до налога в двух вариантах: оплата через Авито Доставку и прямым переводом.</t>
   </si>
   <si>
-    <t xml:space="preserve">    Впишите минимальную цену конкурентов — появится сравнение с рынком. Колонка Y «Цена по рынку (база)» — если цену кита ставим по рынку, а не по наценке.</t>
+    <t xml:space="preserve">    Впишите минимальную цену конкурентов — появится сравнение с рынком. Колонка Y «Цена по рынку» — цена впритык к рынку; если она есть, наценка не применяется.</t>
   </si>
   <si>
     <t xml:space="preserve">4. «Параметры» — наценка, повышение цен (+5%), комиссии, резерв на товар, постоянные расходы и план заказов. Поменяете там — пересчитается всё.</t>
@@ -252,7 +276,7 @@
     <t xml:space="preserve">Статус</t>
   </si>
   <si>
-    <t xml:space="preserve">Цена по рынку (база), ₽</t>
+    <t xml:space="preserve">Цена по рынку, ₽</t>
   </si>
   <si>
     <t xml:space="preserve">TO-01</t>
@@ -804,7 +828,7 @@
     <t xml:space="preserve">Средний чек кита, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Среднее по собранным китам, уже с повышением цен: ТО-кит: Kia Picanto 1.0 / 1.2 (4 390 ₽), VW Jetta (5 090 ₽); ГРМ-кит: Geely Coolray 1.5T (10 490 ₽); Тормоз-кит: Kia Rio 2017–2021 (5 290 ₽), Hyundai Solaris 2017–2022 (5 290 ₽). Замените, когда соберёте больше китов.</t>
+    <t xml:space="preserve">Среднее по собранным китам, уже с повышением цен: ТО-кит: Kia Picanto 1.0 / 1.2 (4 090 ₽), VW Jetta (4 990 ₽); ГРМ-кит: Geely Coolray 1.5T (10 790 ₽); Тормоз-кит: Kia Rio 2017–2021 (5 090 ₽), Hyundai Solaris 2017–2022 (5 090 ₽). Замените, когда соберёте больше китов.</t>
   </si>
   <si>
     <t xml:space="preserve">Средняя стоимость деталей, ₽</t>
@@ -927,10 +951,10 @@
     <t xml:space="preserve">Чтобы цена заканчивалась на …90 (4 700 → 4 690).</t>
   </si>
   <si>
-    <t xml:space="preserve">Повышение цен ко всем китам</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ваше решение: +5% сверху ко всем китам — и к цене по наценке, и к цене по рынку (колонка Y на листе «Киты»). Затем снова округление до …90. Поставьте 0%, чтобы убрать.</t>
+    <t xml:space="preserve">Повышение цен (для китов без цены по рынку)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+5% сверху к цене по наценке, затем округление до …90. Киты с ценой по рынку (колонка Y на листе «Киты») стоят впритык к рынку, повышение к ним не добавляется.</t>
   </si>
   <si>
     <t xml:space="preserve">Комиссия Авито Доставки</t>
@@ -2235,7 +2259,7 @@
         <v/>
       </c>
       <c r="M2" s="11" t="str">
-        <f aca="false">IF(I2="","",CEILING((IF(Y2&lt;&gt;"",Y2,CEILING((I2*(1+Параметры!$B$9*Параметры!$B$10)+K2)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I2="","",IF(Y2&lt;&gt;"",Y2,CEILING((CEILING((I2*(1+Параметры!$B$9*Параметры!$B$10)+K2)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N2" s="12"/>
@@ -2322,7 +2346,7 @@
         <v/>
       </c>
       <c r="M3" s="11" t="str">
-        <f aca="false">IF(I3="","",CEILING((IF(Y3&lt;&gt;"",Y3,CEILING((I3*(1+Параметры!$B$9*Параметры!$B$10)+K3)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I3="","",IF(Y3&lt;&gt;"",Y3,CEILING((CEILING((I3*(1+Параметры!$B$9*Параметры!$B$10)+K3)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N3" s="12"/>
@@ -2409,7 +2433,7 @@
         <v/>
       </c>
       <c r="M4" s="11" t="str">
-        <f aca="false">IF(I4="","",CEILING((IF(Y4&lt;&gt;"",Y4,CEILING((I4*(1+Параметры!$B$9*Параметры!$B$10)+K4)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I4="","",IF(Y4&lt;&gt;"",Y4,CEILING((CEILING((I4*(1+Параметры!$B$9*Параметры!$B$10)+K4)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N4" s="12"/>
@@ -2496,7 +2520,7 @@
         <v/>
       </c>
       <c r="M5" s="11" t="str">
-        <f aca="false">IF(I5="","",CEILING((IF(Y5&lt;&gt;"",Y5,CEILING((I5*(1+Параметры!$B$9*Параметры!$B$10)+K5)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I5="","",IF(Y5&lt;&gt;"",Y5,CEILING((CEILING((I5*(1+Параметры!$B$9*Параметры!$B$10)+K5)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N5" s="12"/>
@@ -2583,7 +2607,7 @@
         <v/>
       </c>
       <c r="M6" s="11" t="str">
-        <f aca="false">IF(I6="","",CEILING((IF(Y6&lt;&gt;"",Y6,CEILING((I6*(1+Параметры!$B$9*Параметры!$B$10)+K6)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I6="","",IF(Y6&lt;&gt;"",Y6,CEILING((CEILING((I6*(1+Параметры!$B$9*Параметры!$B$10)+K6)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N6" s="12"/>
@@ -2670,7 +2694,7 @@
         <v/>
       </c>
       <c r="M7" s="11" t="str">
-        <f aca="false">IF(I7="","",CEILING((IF(Y7&lt;&gt;"",Y7,CEILING((I7*(1+Параметры!$B$9*Параметры!$B$10)+K7)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I7="","",IF(Y7&lt;&gt;"",Y7,CEILING((CEILING((I7*(1+Параметры!$B$9*Параметры!$B$10)+K7)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N7" s="12"/>
@@ -2757,7 +2781,7 @@
         <v/>
       </c>
       <c r="M8" s="11" t="str">
-        <f aca="false">IF(I8="","",CEILING((IF(Y8&lt;&gt;"",Y8,CEILING((I8*(1+Параметры!$B$9*Параметры!$B$10)+K8)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I8="","",IF(Y8&lt;&gt;"",Y8,CEILING((CEILING((I8*(1+Параметры!$B$9*Параметры!$B$10)+K8)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N8" s="12"/>
@@ -2844,7 +2868,7 @@
         <v/>
       </c>
       <c r="M9" s="11" t="str">
-        <f aca="false">IF(I9="","",CEILING((IF(Y9&lt;&gt;"",Y9,CEILING((I9*(1+Параметры!$B$9*Параметры!$B$10)+K9)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I9="","",IF(Y9&lt;&gt;"",Y9,CEILING((CEILING((I9*(1+Параметры!$B$9*Параметры!$B$10)+K9)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N9" s="12"/>
@@ -2931,7 +2955,7 @@
         <v/>
       </c>
       <c r="M10" s="11" t="str">
-        <f aca="false">IF(I10="","",CEILING((IF(Y10&lt;&gt;"",Y10,CEILING((I10*(1+Параметры!$B$9*Параметры!$B$10)+K10)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I10="","",IF(Y10&lt;&gt;"",Y10,CEILING((CEILING((I10*(1+Параметры!$B$9*Параметры!$B$10)+K10)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N10" s="12"/>
@@ -3018,7 +3042,7 @@
         <v/>
       </c>
       <c r="M11" s="11" t="str">
-        <f aca="false">IF(I11="","",CEILING((IF(Y11&lt;&gt;"",Y11,CEILING((I11*(1+Параметры!$B$9*Параметры!$B$10)+K11)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I11="","",IF(Y11&lt;&gt;"",Y11,CEILING((CEILING((I11*(1+Параметры!$B$9*Параметры!$B$10)+K11)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N11" s="12"/>
@@ -3105,7 +3129,7 @@
         <v/>
       </c>
       <c r="M12" s="11" t="str">
-        <f aca="false">IF(I12="","",CEILING((IF(Y12&lt;&gt;"",Y12,CEILING((I12*(1+Параметры!$B$9*Параметры!$B$10)+K12)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I12="","",IF(Y12&lt;&gt;"",Y12,CEILING((CEILING((I12*(1+Параметры!$B$9*Параметры!$B$10)+K12)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N12" s="12"/>
@@ -3192,7 +3216,7 @@
         <v/>
       </c>
       <c r="M13" s="11" t="str">
-        <f aca="false">IF(I13="","",CEILING((IF(Y13&lt;&gt;"",Y13,CEILING((I13*(1+Параметры!$B$9*Параметры!$B$10)+K13)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I13="","",IF(Y13&lt;&gt;"",Y13,CEILING((CEILING((I13*(1+Параметры!$B$9*Параметры!$B$10)+K13)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N13" s="12"/>
@@ -3279,7 +3303,7 @@
         <v/>
       </c>
       <c r="M14" s="11" t="str">
-        <f aca="false">IF(I14="","",CEILING((IF(Y14&lt;&gt;"",Y14,CEILING((I14*(1+Параметры!$B$9*Параметры!$B$10)+K14)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I14="","",IF(Y14&lt;&gt;"",Y14,CEILING((CEILING((I14*(1+Параметры!$B$9*Параметры!$B$10)+K14)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N14" s="12"/>
@@ -3322,7 +3346,9 @@
       <c r="X14" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="Y14" s="12"/>
+      <c r="Y14" s="12" t="n">
+        <v>4090</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
@@ -3366,7 +3392,7 @@
         <v/>
       </c>
       <c r="M15" s="11" t="str">
-        <f aca="false">IF(I15="","",CEILING((IF(Y15&lt;&gt;"",Y15,CEILING((I15*(1+Параметры!$B$9*Параметры!$B$10)+K15)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I15="","",IF(Y15&lt;&gt;"",Y15,CEILING((CEILING((I15*(1+Параметры!$B$9*Параметры!$B$10)+K15)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N15" s="12"/>
@@ -3409,7 +3435,9 @@
       <c r="X15" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="Y15" s="12"/>
+      <c r="Y15" s="12" t="n">
+        <v>4990</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
@@ -3453,7 +3481,7 @@
         <v/>
       </c>
       <c r="M16" s="11" t="str">
-        <f aca="false">IF(I16="","",CEILING((IF(Y16&lt;&gt;"",Y16,CEILING((I16*(1+Параметры!$B$9*Параметры!$B$10)+K16)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I16="","",IF(Y16&lt;&gt;"",Y16,CEILING((CEILING((I16*(1+Параметры!$B$9*Параметры!$B$10)+K16)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N16" s="12"/>
@@ -3540,7 +3568,7 @@
         <v/>
       </c>
       <c r="M17" s="11" t="str">
-        <f aca="false">IF(I17="","",CEILING((IF(Y17&lt;&gt;"",Y17,CEILING((I17*(1+Параметры!$B$9*Параметры!$B$10)+K17)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I17="","",IF(Y17&lt;&gt;"",Y17,CEILING((CEILING((I17*(1+Параметры!$B$9*Параметры!$B$10)+K17)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N17" s="12"/>
@@ -3627,7 +3655,7 @@
         <v/>
       </c>
       <c r="M18" s="11" t="str">
-        <f aca="false">IF(I18="","",CEILING((IF(Y18&lt;&gt;"",Y18,CEILING((I18*(1+Параметры!$B$9*Параметры!$B$10)+K18)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I18="","",IF(Y18&lt;&gt;"",Y18,CEILING((CEILING((I18*(1+Параметры!$B$9*Параметры!$B$10)+K18)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N18" s="12"/>
@@ -3714,7 +3742,7 @@
         <v/>
       </c>
       <c r="M19" s="11" t="str">
-        <f aca="false">IF(I19="","",CEILING((IF(Y19&lt;&gt;"",Y19,CEILING((I19*(1+Параметры!$B$9*Параметры!$B$10)+K19)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I19="","",IF(Y19&lt;&gt;"",Y19,CEILING((CEILING((I19*(1+Параметры!$B$9*Параметры!$B$10)+K19)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N19" s="12"/>
@@ -3801,7 +3829,7 @@
         <v/>
       </c>
       <c r="M20" s="11" t="str">
-        <f aca="false">IF(I20="","",CEILING((IF(Y20&lt;&gt;"",Y20,CEILING((I20*(1+Параметры!$B$9*Параметры!$B$10)+K20)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I20="","",IF(Y20&lt;&gt;"",Y20,CEILING((CEILING((I20*(1+Параметры!$B$9*Параметры!$B$10)+K20)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N20" s="12"/>
@@ -3888,7 +3916,7 @@
         <v/>
       </c>
       <c r="M21" s="11" t="str">
-        <f aca="false">IF(I21="","",CEILING((IF(Y21&lt;&gt;"",Y21,CEILING((I21*(1+Параметры!$B$9*Параметры!$B$10)+K21)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I21="","",IF(Y21&lt;&gt;"",Y21,CEILING((CEILING((I21*(1+Параметры!$B$9*Параметры!$B$10)+K21)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N21" s="12"/>
@@ -3975,7 +4003,7 @@
         <v/>
       </c>
       <c r="M22" s="11" t="str">
-        <f aca="false">IF(I22="","",CEILING((IF(Y22&lt;&gt;"",Y22,CEILING((I22*(1+Параметры!$B$9*Параметры!$B$10)+K22)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I22="","",IF(Y22&lt;&gt;"",Y22,CEILING((CEILING((I22*(1+Параметры!$B$9*Параметры!$B$10)+K22)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N22" s="12"/>
@@ -4062,7 +4090,7 @@
         <v/>
       </c>
       <c r="M23" s="11" t="str">
-        <f aca="false">IF(I23="","",CEILING((IF(Y23&lt;&gt;"",Y23,CEILING((I23*(1+Параметры!$B$9*Параметры!$B$10)+K23)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I23="","",IF(Y23&lt;&gt;"",Y23,CEILING((CEILING((I23*(1+Параметры!$B$9*Параметры!$B$10)+K23)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N23" s="12"/>
@@ -4149,7 +4177,7 @@
         <v/>
       </c>
       <c r="M24" s="11" t="str">
-        <f aca="false">IF(I24="","",CEILING((IF(Y24&lt;&gt;"",Y24,CEILING((I24*(1+Параметры!$B$9*Параметры!$B$10)+K24)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I24="","",IF(Y24&lt;&gt;"",Y24,CEILING((CEILING((I24*(1+Параметры!$B$9*Параметры!$B$10)+K24)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N24" s="12"/>
@@ -4236,7 +4264,7 @@
         <v/>
       </c>
       <c r="M25" s="11" t="str">
-        <f aca="false">IF(I25="","",CEILING((IF(Y25&lt;&gt;"",Y25,CEILING((I25*(1+Параметры!$B$9*Параметры!$B$10)+K25)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I25="","",IF(Y25&lt;&gt;"",Y25,CEILING((CEILING((I25*(1+Параметры!$B$9*Параметры!$B$10)+K25)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N25" s="12"/>
@@ -4323,7 +4351,7 @@
         <v/>
       </c>
       <c r="M26" s="11" t="str">
-        <f aca="false">IF(I26="","",CEILING((IF(Y26&lt;&gt;"",Y26,CEILING((I26*(1+Параметры!$B$9*Параметры!$B$10)+K26)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I26="","",IF(Y26&lt;&gt;"",Y26,CEILING((CEILING((I26*(1+Параметры!$B$9*Параметры!$B$10)+K26)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N26" s="12"/>
@@ -4367,7 +4395,7 @@
         <v>48</v>
       </c>
       <c r="Y26" s="12" t="n">
-        <v>9990</v>
+        <v>10790</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4412,7 +4440,7 @@
         <v/>
       </c>
       <c r="M27" s="11" t="str">
-        <f aca="false">IF(I27="","",CEILING((IF(Y27&lt;&gt;"",Y27,CEILING((I27*(1+Параметры!$B$9*Параметры!$B$10)+K27)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I27="","",IF(Y27&lt;&gt;"",Y27,CEILING((CEILING((I27*(1+Параметры!$B$9*Параметры!$B$10)+K27)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N27" s="12"/>
@@ -4456,7 +4484,7 @@
         <v>48</v>
       </c>
       <c r="Y27" s="12" t="n">
-        <v>4990</v>
+        <v>5090</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4501,7 +4529,7 @@
         <v/>
       </c>
       <c r="M28" s="11" t="str">
-        <f aca="false">IF(I28="","",CEILING((IF(Y28&lt;&gt;"",Y28,CEILING((I28*(1+Параметры!$B$9*Параметры!$B$10)+K28)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5))*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5)</f>
+        <f aca="false">IF(I28="","",IF(Y28&lt;&gt;"",Y28,CEILING((CEILING((I28*(1+Параметры!$B$9*Параметры!$B$10)+K28)*(1+Параметры!$B$2),Параметры!$B$4)-Параметры!$B$5)*(1+Параметры!$B$6),Параметры!$B$4)-Параметры!$B$5))</f>
         <v/>
       </c>
       <c r="N28" s="12"/>
@@ -4545,7 +4573,7 @@
         <v>48</v>
       </c>
       <c r="Y28" s="12" t="n">
-        <v>4990</v>
+        <v>5090</v>
       </c>
     </row>
   </sheetData>
@@ -12849,13 +12877,13 @@
         <v>222</v>
       </c>
       <c r="B4" s="12" t="n">
-        <v>4740</v>
+        <v>4540</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>10490</v>
+        <v>10790</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>5290</v>
+        <v>5090</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>223</v>
@@ -12977,15 +13005,15 @@
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">IF(B4="","",B4-(B5+Параметры!$B$3)-$B$6*B4*Параметры!$B$7-(1-$B$6)*(B4*Параметры!$B$11+Параметры!$B$12)-Параметры!$B$8-B5*Параметры!$B$9)</f>
-        <v>806.0155</v>
+        <v>613.2155</v>
       </c>
       <c r="C10" s="11" t="n">
         <f aca="false">IF(C4="","",C4-(C5+Параметры!$B$3)-$B$6*C4*Параметры!$B$7-(1-$B$6)*(C4*Параметры!$B$11+Параметры!$B$12)-Параметры!$B$8-C5*Параметры!$B$9)</f>
-        <v>2473.3185</v>
+        <v>2762.5185</v>
       </c>
       <c r="D10" s="11" t="n">
         <f aca="false">IF(D4="","",D4-(D5+Параметры!$B$3)-$B$6*D4*Параметры!$B$7-(1-$B$6)*(D4*Параметры!$B$11+Параметры!$B$12)-Параметры!$B$8-D5*Параметры!$B$9)</f>
-        <v>1063.73</v>
+        <v>870.93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12994,15 +13022,15 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">IF(B10="","",IF(B10&lt;=0,"не окупается",ROUNDUP($B$9/B10,0)))</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C11" s="6" t="n">
         <f aca="false">IF(C10="","",IF(C10&lt;=0,"не окупается",ROUNDUP($B$9/C10,0)))</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">IF(D10="","",IF(D10&lt;=0,"не окупается",ROUNDUP($B$9/D10,0)))</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>234</v>
@@ -13076,7 +13104,7 @@
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">N(B14)*N($B$4)+N(C14)*N($C$4)+N(D14)*N($D$4)</f>
-        <v>94800</v>
+        <v>90800</v>
       </c>
       <c r="F14" s="9" t="n">
         <f aca="false">N(B14)*(N($B$5)+Параметры!$B$3)+N(C14)*(N($C$5)+Параметры!$B$3)+N(D14)*(N($D$5)+Параметры!$B$3)</f>
@@ -13084,11 +13112,11 @@
       </c>
       <c r="G14" s="9" t="n">
         <f aca="false">$B$6*E14*Параметры!$B$7</f>
-        <v>3081</v>
+        <v>2951</v>
       </c>
       <c r="H14" s="9" t="n">
         <f aca="false">(1-$B$6)*E14*Параметры!$B$11</f>
-        <v>331.8</v>
+        <v>317.8</v>
       </c>
       <c r="I14" s="9" t="n">
         <f aca="false">(B14+C14+D14)*Параметры!$B$8</f>
@@ -13108,11 +13136,11 @@
       </c>
       <c r="M14" s="11" t="n">
         <f aca="false">E14-SUM(F14:L14)</f>
-        <v>3337.31</v>
+        <v>-518.690000000002</v>
       </c>
       <c r="N14" s="9" t="n">
         <f aca="false">IF((B14+C14+D14)=0,"",M14/(B14+C14+D14))</f>
-        <v>166.8655</v>
+        <v>-25.9345000000001</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13130,7 +13158,7 @@
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">N(B15)*N($B$4)+N(C15)*N($C$4)+N(D15)*N($D$4)</f>
-        <v>104900</v>
+        <v>107900</v>
       </c>
       <c r="F15" s="9" t="n">
         <f aca="false">N(B15)*(N($B$5)+Параметры!$B$3)+N(C15)*(N($C$5)+Параметры!$B$3)+N(D15)*(N($D$5)+Параметры!$B$3)</f>
@@ -13138,11 +13166,11 @@
       </c>
       <c r="G15" s="9" t="n">
         <f aca="false">$B$6*E15*Параметры!$B$7</f>
-        <v>3409.25</v>
+        <v>3506.75</v>
       </c>
       <c r="H15" s="9" t="n">
         <f aca="false">(1-$B$6)*E15*Параметры!$B$11</f>
-        <v>367.15</v>
+        <v>377.65</v>
       </c>
       <c r="I15" s="9" t="n">
         <f aca="false">(B15+C15+D15)*Параметры!$B$8</f>
@@ -13162,11 +13190,11 @@
       </c>
       <c r="M15" s="11" t="n">
         <f aca="false">E15-SUM(F15:L15)</f>
-        <v>11950.185</v>
+        <v>14842.185</v>
       </c>
       <c r="N15" s="9" t="n">
         <f aca="false">IF((B15+C15+D15)=0,"",M15/(B15+C15+D15))</f>
-        <v>1195.0185</v>
+        <v>1484.2185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13184,7 +13212,7 @@
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">N(B16)*N($B$4)+N(C16)*N($C$4)+N(D16)*N($D$4)</f>
-        <v>52900</v>
+        <v>50900</v>
       </c>
       <c r="F16" s="9" t="n">
         <f aca="false">N(B16)*(N($B$5)+Параметры!$B$3)+N(C16)*(N($C$5)+Параметры!$B$3)+N(D16)*(N($D$5)+Параметры!$B$3)</f>
@@ -13192,11 +13220,11 @@
       </c>
       <c r="G16" s="9" t="n">
         <f aca="false">$B$6*E16*Параметры!$B$7</f>
-        <v>1719.25</v>
+        <v>1654.25</v>
       </c>
       <c r="H16" s="9" t="n">
         <f aca="false">(1-$B$6)*E16*Параметры!$B$11</f>
-        <v>185.15</v>
+        <v>178.15</v>
       </c>
       <c r="I16" s="9" t="n">
         <f aca="false">(B16+C16+D16)*Параметры!$B$8</f>
@@ -13216,11 +13244,11 @@
       </c>
       <c r="M16" s="11" t="n">
         <f aca="false">E16-SUM(F16:L16)</f>
-        <v>-2145.7</v>
+        <v>-4073.7</v>
       </c>
       <c r="N16" s="9" t="n">
         <f aca="false">IF((B16+C16+D16)=0,"",M16/(B16+C16+D16))</f>
-        <v>-214.57</v>
+        <v>-407.37</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13238,7 +13266,7 @@
       </c>
       <c r="E17" s="9" t="n">
         <f aca="false">N(B17)*N($B$4)+N(C17)*N($C$4)+N(D17)*N($D$4)</f>
-        <v>126300</v>
+        <v>124800</v>
       </c>
       <c r="F17" s="9" t="n">
         <f aca="false">N(B17)*(N($B$5)+Параметры!$B$3)+N(C17)*(N($C$5)+Параметры!$B$3)+N(D17)*(N($D$5)+Параметры!$B$3)</f>
@@ -13246,11 +13274,11 @@
       </c>
       <c r="G17" s="9" t="n">
         <f aca="false">$B$6*E17*Параметры!$B$7</f>
-        <v>4104.75</v>
+        <v>4056</v>
       </c>
       <c r="H17" s="9" t="n">
         <f aca="false">(1-$B$6)*E17*Параметры!$B$11</f>
-        <v>442.05</v>
+        <v>436.8</v>
       </c>
       <c r="I17" s="9" t="n">
         <f aca="false">(B17+C17+D17)*Параметры!$B$8</f>
@@ -13270,11 +13298,11 @@
       </c>
       <c r="M17" s="11" t="n">
         <f aca="false">E17-SUM(F17:L17)</f>
-        <v>12962.3975</v>
+        <v>11516.3975</v>
       </c>
       <c r="N17" s="9" t="n">
         <f aca="false">IF((B17+C17+D17)=0,"",M17/(B17+C17+D17))</f>
-        <v>648.119875</v>
+        <v>575.819875</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13292,7 +13320,7 @@
       </c>
       <c r="E18" s="9" t="n">
         <f aca="false">N(B18)*N($B$4)+N(C18)*N($C$4)+N(D18)*N($D$4)</f>
-        <v>252600</v>
+        <v>249600</v>
       </c>
       <c r="F18" s="9" t="n">
         <f aca="false">N(B18)*(N($B$5)+Параметры!$B$3)+N(C18)*(N($C$5)+Параметры!$B$3)+N(D18)*(N($D$5)+Параметры!$B$3)</f>
@@ -13300,11 +13328,11 @@
       </c>
       <c r="G18" s="9" t="n">
         <f aca="false">$B$6*E18*Параметры!$B$7</f>
-        <v>8209.5</v>
+        <v>8112</v>
       </c>
       <c r="H18" s="9" t="n">
         <f aca="false">(1-$B$6)*E18*Параметры!$B$11</f>
-        <v>884.1</v>
+        <v>873.6</v>
       </c>
       <c r="I18" s="9" t="n">
         <f aca="false">(B18+C18+D18)*Параметры!$B$8</f>
@@ -13324,11 +13352,11 @@
       </c>
       <c r="M18" s="11" t="n">
         <f aca="false">E18-SUM(F18:L18)</f>
-        <v>38707.795</v>
+        <v>35815.795</v>
       </c>
       <c r="N18" s="9" t="n">
         <f aca="false">IF((B18+C18+D18)=0,"",M18/(B18+C18+D18))</f>
-        <v>967.694875</v>
+        <v>895.394875</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13346,7 +13374,7 @@
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">N(B19)*N($B$4)+N(C19)*N($C$4)+N(D19)*N($D$4)</f>
-        <v>378900</v>
+        <v>374400</v>
       </c>
       <c r="F19" s="9" t="n">
         <f aca="false">N(B19)*(N($B$5)+Параметры!$B$3)+N(C19)*(N($C$5)+Параметры!$B$3)+N(D19)*(N($D$5)+Параметры!$B$3)</f>
@@ -13354,11 +13382,11 @@
       </c>
       <c r="G19" s="9" t="n">
         <f aca="false">$B$6*E19*Параметры!$B$7</f>
-        <v>12314.25</v>
+        <v>12168</v>
       </c>
       <c r="H19" s="9" t="n">
         <f aca="false">(1-$B$6)*E19*Параметры!$B$11</f>
-        <v>1326.15</v>
+        <v>1310.4</v>
       </c>
       <c r="I19" s="9" t="n">
         <f aca="false">(B19+C19+D19)*Параметры!$B$8</f>
@@ -13378,11 +13406,11 @@
       </c>
       <c r="M19" s="11" t="n">
         <f aca="false">E19-SUM(F19:L19)</f>
-        <v>64453.1925</v>
+        <v>60115.1925</v>
       </c>
       <c r="N19" s="9" t="n">
         <f aca="false">IF((B19+C19+D19)=0,"",M19/(B19+C19+D19))</f>
-        <v>1074.219875</v>
+        <v>1001.919875</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13400,7 +13428,7 @@
       </c>
       <c r="E20" s="9" t="n">
         <f aca="false">N(B20)*N($B$4)+N(C20)*N($C$4)+N(D20)*N($D$4)</f>
-        <v>552600</v>
+        <v>544600</v>
       </c>
       <c r="F20" s="9" t="n">
         <f aca="false">N(B20)*(N($B$5)+Параметры!$B$3)+N(C20)*(N($C$5)+Параметры!$B$3)+N(D20)*(N($D$5)+Параметры!$B$3)</f>
@@ -13408,11 +13436,11 @@
       </c>
       <c r="G20" s="9" t="n">
         <f aca="false">$B$6*E20*Параметры!$B$7</f>
-        <v>17959.5</v>
+        <v>17699.5</v>
       </c>
       <c r="H20" s="9" t="n">
         <f aca="false">(1-$B$6)*E20*Параметры!$B$11</f>
-        <v>1934.1</v>
+        <v>1906.1</v>
       </c>
       <c r="I20" s="9" t="n">
         <f aca="false">(B20+C20+D20)*Параметры!$B$8</f>
@@ -13432,11 +13460,11 @@
       </c>
       <c r="M20" s="11" t="n">
         <f aca="false">E20-SUM(F20:L20)</f>
-        <v>98258.745</v>
+        <v>90546.745</v>
       </c>
       <c r="N20" s="9" t="n">
         <f aca="false">IF((B20+C20+D20)=0,"",M20/(B20+C20+D20))</f>
-        <v>1091.76383333333</v>
+        <v>1006.07494444444</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>